<commit_message>
Google Sheets: suite passes 188/188; fix log OEE colours in Sheets
Sheets ignores conditional formats that reference another sheet, so the
Production Log OEE colours now use a hidden same-sheet copy of the target.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FtnizgcUQQWB874QqXt4YR
</commit_message>
<xml_diff>
--- a/products/manufacturing-templates/dist/Downtime-Log-and-Pareto.xlsx
+++ b/products/manufacturing-templates/dist/Downtime-Log-and-Pareto.xlsx
@@ -859,8 +859,8 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="87713356"/>
-        <c:axId val="99447213"/>
+        <c:axId val="7198020"/>
+        <c:axId val="6383468"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -996,11 +996,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="59086187"/>
-        <c:axId val="2429952"/>
+        <c:axId val="62506310"/>
+        <c:axId val="68067979"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="87713356"/>
+        <c:axId val="7198020"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1032,7 +1032,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="99447213"/>
+        <c:crossAx val="6383468"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1040,7 +1040,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="99447213"/>
+        <c:axId val="6383468"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1116,12 +1116,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="87713356"/>
+        <c:crossAx val="7198020"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:catAx>
-        <c:axId val="59086187"/>
+        <c:axId val="62506310"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1153,7 +1153,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2429952"/>
+        <c:crossAx val="68067979"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1161,7 +1161,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="2429952"/>
+        <c:axId val="68067979"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -1229,7 +1229,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="59086187"/>
+        <c:crossAx val="62506310"/>
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>

</xml_diff>

<commit_message>
Google Sheets: suite passes 188/188; fix log OEE colours in Sheets (#44)
Sheets ignores conditional formats that reference another sheet, so the
Production Log OEE colours now use a hidden same-sheet copy of the target.


Claude-Session: https://claude.ai/code/session_01FtnizgcUQQWB874QqXt4YR

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/products/manufacturing-templates/dist/Downtime-Log-and-Pareto.xlsx
+++ b/products/manufacturing-templates/dist/Downtime-Log-and-Pareto.xlsx
@@ -859,8 +859,8 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="87713356"/>
-        <c:axId val="99447213"/>
+        <c:axId val="7198020"/>
+        <c:axId val="6383468"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -996,11 +996,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="59086187"/>
-        <c:axId val="2429952"/>
+        <c:axId val="62506310"/>
+        <c:axId val="68067979"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="87713356"/>
+        <c:axId val="7198020"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1032,7 +1032,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="99447213"/>
+        <c:crossAx val="6383468"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1040,7 +1040,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="99447213"/>
+        <c:axId val="6383468"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1116,12 +1116,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="87713356"/>
+        <c:crossAx val="7198020"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:catAx>
-        <c:axId val="59086187"/>
+        <c:axId val="62506310"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1153,7 +1153,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2429952"/>
+        <c:crossAx val="68067979"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1161,7 +1161,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="2429952"/>
+        <c:axId val="68067979"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -1229,7 +1229,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="59086187"/>
+        <c:crossAx val="62506310"/>
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>

</xml_diff>

<commit_message>
Hold: Pareto chart fix for Excel, plus Excel for the web results (not for merge yet)
- Pareto line plots a helper column that carries the last cumulative % forward,
  so empty rows no longer plot as 0 in Excel. Found uncommitted in the workspace;
  passes LibreOffice 188/188, not yet checked in Excel.
- Excel for the web: 188/188 suite checks pass (results-excel-web.json).

On hold pending the owner's decision in #48 (tripwire). No PR opened.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FtnizgcUQQWB874QqXt4YR
</commit_message>
<xml_diff>
--- a/products/manufacturing-templates/dist/Downtime-Log-and-Pareto.xlsx
+++ b/products/manufacturing-templates/dist/Downtime-Log-and-Pareto.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="86">
   <si>
     <t xml:space="preserve">Downtime Log &amp; Pareto</t>
   </si>
@@ -302,7 +302,7 @@
     <numFmt numFmtId="170" formatCode="0%"/>
     <numFmt numFmtId="171" formatCode="0.0"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="18">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -410,6 +410,12 @@
       <family val="2"/>
     </font>
     <font>
+      <sz val="8"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
@@ -498,7 +504,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="33">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -583,6 +589,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -596,6 +606,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -859,8 +873,8 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="7198020"/>
-        <c:axId val="6383468"/>
+        <c:axId val="30367123"/>
+        <c:axId val="10482130"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -870,7 +884,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>Pareto!F8</c:f>
+              <c:f>Pareto!M8</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -964,7 +978,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Pareto!$F$9:$F$20</c:f>
+              <c:f>Pareto!$M$9:$M$20</c:f>
               <c:numCache>
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="12"/>
@@ -983,6 +997,27 @@
                 <c:pt idx="4">
                   <c:v>1</c:v>
                 </c:pt>
+                <c:pt idx="5">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>1</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -996,11 +1031,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="62506310"/>
-        <c:axId val="68067979"/>
+        <c:axId val="42842550"/>
+        <c:axId val="48986869"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="7198020"/>
+        <c:axId val="30367123"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1019,11 +1054,11 @@
           </a:ln>
         </c:spPr>
         <c:txPr>
-          <a:bodyPr/>
+          <a:bodyPr rot="-2700000"/>
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+              <a:defRPr b="0" sz="800" spc="-1" strike="noStrike">
                 <a:solidFill>
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
@@ -1032,7 +1067,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="6383468"/>
+        <c:crossAx val="10482130"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1040,7 +1075,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="6383468"/>
+        <c:axId val="10482130"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1116,16 +1151,16 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="7198020"/>
+        <c:crossAx val="30367123"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:catAx>
-        <c:axId val="62506310"/>
+        <c:axId val="42842550"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
-        <c:delete val="0"/>
+        <c:delete val="1"/>
         <c:axPos val="t"/>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
@@ -1153,15 +1188,14 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="68067979"/>
-        <c:crosses val="autoZero"/>
+        <c:crossAx val="48986869"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="68067979"/>
+        <c:axId val="48986869"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -1229,7 +1263,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="62506310"/>
+        <c:crossAx val="42842550"/>
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1264,7 +1298,7 @@
         </a:p>
       </c:txPr>
     </c:legend>
-    <c:plotVisOnly val="1"/>
+    <c:plotVisOnly val="0"/>
     <c:dispBlanksAs val="gap"/>
   </c:chart>
   <c:spPr>
@@ -1285,16 +1319,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>7</xdr:col>
+      <xdr:col>13</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>130680</xdr:rowOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>340200</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>23</xdr:col>
-      <xdr:colOff>261720</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>112680</xdr:rowOff>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>473400</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>131760</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1302,7 +1336,7 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="7518960" y="380880"/>
+        <a:off x="7730640" y="1733400"/>
         <a:ext cx="7199640" cy="3239640"/>
       </xdr:xfrm>
       <a:graphic>
@@ -24290,7 +24324,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L38"/>
+  <dimension ref="A1:M38"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
@@ -24304,6 +24338,7 @@
     <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="10" min="10" style="0" width="11"/>
     <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="11" min="11" style="0" width="9"/>
     <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="12" min="12" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="13" min="13" style="0" width="13"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -24394,16 +24429,19 @@
       <c r="L8" s="20" t="s">
         <v>78</v>
       </c>
+      <c r="M8" s="21" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="21" t="n">
+      <c r="A9" s="22" t="n">
         <v>1</v>
       </c>
       <c r="B9" s="10" t="str">
         <f aca="false">IF(INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A9),$L$9:$L$38,0))&lt;=0,"",INDEX($I$9:$I$38,MATCH(LARGE($L$9:$L$38,A9),$L$9:$L$38,0)))</f>
         <v>Mechanical breakdown</v>
       </c>
-      <c r="C9" s="22" t="n">
+      <c r="C9" s="23" t="n">
         <f aca="false">IF(B9="","",INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A9),$L$9:$L$38,0)))</f>
         <v>100</v>
       </c>
@@ -24411,40 +24449,44 @@
         <f aca="false">IF(B9="","",INDEX($K$9:$K$38,MATCH(LARGE($L$9:$L$38,A9),$L$9:$L$38,0)))</f>
         <v>2</v>
       </c>
-      <c r="E9" s="23" t="n">
+      <c r="E9" s="24" t="n">
         <f aca="false">IF(OR(B9="",$B$6=0),"",C9/$B$6)</f>
         <v>0.392156862745098</v>
       </c>
-      <c r="F9" s="23" t="n">
+      <c r="F9" s="24" t="n">
         <f aca="false">IF(OR(B9="",$B$6=0),"",SUM($C$9:C9)/$B$6)</f>
         <v>0.392156862745098</v>
       </c>
-      <c r="I9" s="24" t="str">
+      <c r="I9" s="25" t="str">
         <f aca="false">IF(Setup!D5="","",IF(SUMPRODUCT(--(Setup!$D$4:D4=Setup!D5))&gt;0,"",Setup!D5))</f>
         <v>Mechanical breakdown</v>
       </c>
-      <c r="J9" s="24" t="n">
+      <c r="J9" s="25" t="n">
         <f aca="false">IF(I9="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I9)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0),'Downtime Log'!$G$5:$G$1004))</f>
         <v>100</v>
       </c>
-      <c r="K9" s="24" t="n">
+      <c r="K9" s="25" t="n">
         <f aca="false">IF(I9="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I9)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>2</v>
       </c>
-      <c r="L9" s="24" t="n">
+      <c r="L9" s="25" t="n">
         <f aca="false">IF(I9="",-1,J9+(34-1)/1000000)</f>
         <v>100.000033</v>
       </c>
+      <c r="M9" s="26" t="n">
+        <f aca="false">IF(B9&lt;&gt;"",F9,"")</f>
+        <v>0.392156862745098</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="21" t="n">
+      <c r="A10" s="22" t="n">
         <v>2</v>
       </c>
       <c r="B10" s="10" t="str">
         <f aca="false">IF(INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A10),$L$9:$L$38,0))&lt;=0,"",INDEX($I$9:$I$38,MATCH(LARGE($L$9:$L$38,A10),$L$9:$L$38,0)))</f>
         <v>Changeover / setup</v>
       </c>
-      <c r="C10" s="22" t="n">
+      <c r="C10" s="23" t="n">
         <f aca="false">IF(B10="","",INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A10),$L$9:$L$38,0)))</f>
         <v>65</v>
       </c>
@@ -24452,40 +24494,44 @@
         <f aca="false">IF(B10="","",INDEX($K$9:$K$38,MATCH(LARGE($L$9:$L$38,A10),$L$9:$L$38,0)))</f>
         <v>2</v>
       </c>
-      <c r="E10" s="23" t="n">
+      <c r="E10" s="24" t="n">
         <f aca="false">IF(OR(B10="",$B$6=0),"",C10/$B$6)</f>
         <v>0.254901960784314</v>
       </c>
-      <c r="F10" s="23" t="n">
+      <c r="F10" s="24" t="n">
         <f aca="false">IF(OR(B10="",$B$6=0),"",SUM($C$9:C10)/$B$6)</f>
         <v>0.647058823529412</v>
       </c>
-      <c r="I10" s="24" t="str">
+      <c r="I10" s="25" t="str">
         <f aca="false">IF(Setup!D6="","",IF(SUMPRODUCT(--(Setup!$D$4:D5=Setup!D6))&gt;0,"",Setup!D6))</f>
         <v>Electrical / controls fault</v>
       </c>
-      <c r="J10" s="24" t="n">
+      <c r="J10" s="25" t="n">
         <f aca="false">IF(I10="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I10)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0),'Downtime Log'!$G$5:$G$1004))</f>
         <v>0</v>
       </c>
-      <c r="K10" s="24" t="n">
+      <c r="K10" s="25" t="n">
         <f aca="false">IF(I10="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I10)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>0</v>
       </c>
-      <c r="L10" s="24" t="n">
+      <c r="L10" s="25" t="n">
         <f aca="false">IF(I10="",-1,J10+(34-2)/1000000)</f>
         <v>3.2E-005</v>
       </c>
+      <c r="M10" s="26" t="n">
+        <f aca="false">IF(B10&lt;&gt;"",F10,M9)</f>
+        <v>0.647058823529412</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="21" t="n">
+      <c r="A11" s="22" t="n">
         <v>3</v>
       </c>
       <c r="B11" s="10" t="str">
         <f aca="false">IF(INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A11),$L$9:$L$38,0))&lt;=0,"",INDEX($I$9:$I$38,MATCH(LARGE($L$9:$L$38,A11),$L$9:$L$38,0)))</f>
         <v>Tooling failure</v>
       </c>
-      <c r="C11" s="22" t="n">
+      <c r="C11" s="23" t="n">
         <f aca="false">IF(B11="","",INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A11),$L$9:$L$38,0)))</f>
         <v>60</v>
       </c>
@@ -24493,40 +24539,44 @@
         <f aca="false">IF(B11="","",INDEX($K$9:$K$38,MATCH(LARGE($L$9:$L$38,A11),$L$9:$L$38,0)))</f>
         <v>1</v>
       </c>
-      <c r="E11" s="23" t="n">
+      <c r="E11" s="24" t="n">
         <f aca="false">IF(OR(B11="",$B$6=0),"",C11/$B$6)</f>
         <v>0.235294117647059</v>
       </c>
-      <c r="F11" s="23" t="n">
+      <c r="F11" s="24" t="n">
         <f aca="false">IF(OR(B11="",$B$6=0),"",SUM($C$9:C11)/$B$6)</f>
         <v>0.882352941176471</v>
       </c>
-      <c r="I11" s="24" t="str">
+      <c r="I11" s="25" t="str">
         <f aca="false">IF(Setup!D7="","",IF(SUMPRODUCT(--(Setup!$D$4:D6=Setup!D7))&gt;0,"",Setup!D7))</f>
         <v>Tooling failure</v>
       </c>
-      <c r="J11" s="24" t="n">
+      <c r="J11" s="25" t="n">
         <f aca="false">IF(I11="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I11)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0),'Downtime Log'!$G$5:$G$1004))</f>
         <v>60</v>
       </c>
-      <c r="K11" s="24" t="n">
+      <c r="K11" s="25" t="n">
         <f aca="false">IF(I11="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I11)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>1</v>
       </c>
-      <c r="L11" s="24" t="n">
+      <c r="L11" s="25" t="n">
         <f aca="false">IF(I11="",-1,J11+(34-3)/1000000)</f>
         <v>60.000031</v>
       </c>
+      <c r="M11" s="26" t="n">
+        <f aca="false">IF(B11&lt;&gt;"",F11,M10)</f>
+        <v>0.882352941176471</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="21" t="n">
+      <c r="A12" s="22" t="n">
         <v>4</v>
       </c>
       <c r="B12" s="10" t="str">
         <f aca="false">IF(INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A12),$L$9:$L$38,0))&lt;=0,"",INDEX($I$9:$I$38,MATCH(LARGE($L$9:$L$38,A12),$L$9:$L$38,0)))</f>
         <v>Waiting for material</v>
       </c>
-      <c r="C12" s="22" t="n">
+      <c r="C12" s="23" t="n">
         <f aca="false">IF(B12="","",INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A12),$L$9:$L$38,0)))</f>
         <v>15</v>
       </c>
@@ -24534,40 +24584,44 @@
         <f aca="false">IF(B12="","",INDEX($K$9:$K$38,MATCH(LARGE($L$9:$L$38,A12),$L$9:$L$38,0)))</f>
         <v>1</v>
       </c>
-      <c r="E12" s="23" t="n">
+      <c r="E12" s="24" t="n">
         <f aca="false">IF(OR(B12="",$B$6=0),"",C12/$B$6)</f>
         <v>0.0588235294117647</v>
       </c>
-      <c r="F12" s="23" t="n">
+      <c r="F12" s="24" t="n">
         <f aca="false">IF(OR(B12="",$B$6=0),"",SUM($C$9:C12)/$B$6)</f>
         <v>0.941176470588235</v>
       </c>
-      <c r="I12" s="24" t="str">
+      <c r="I12" s="25" t="str">
         <f aca="false">IF(Setup!D8="","",IF(SUMPRODUCT(--(Setup!$D$4:D7=Setup!D8))&gt;0,"",Setup!D8))</f>
         <v>Changeover / setup</v>
       </c>
-      <c r="J12" s="24" t="n">
+      <c r="J12" s="25" t="n">
         <f aca="false">IF(I12="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I12)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0),'Downtime Log'!$G$5:$G$1004))</f>
         <v>65</v>
       </c>
-      <c r="K12" s="24" t="n">
+      <c r="K12" s="25" t="n">
         <f aca="false">IF(I12="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I12)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>2</v>
       </c>
-      <c r="L12" s="24" t="n">
+      <c r="L12" s="25" t="n">
         <f aca="false">IF(I12="",-1,J12+(34-4)/1000000)</f>
         <v>65.00003</v>
       </c>
+      <c r="M12" s="26" t="n">
+        <f aca="false">IF(B12&lt;&gt;"",F12,M11)</f>
+        <v>0.941176470588235</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="21" t="n">
+      <c r="A13" s="22" t="n">
         <v>5</v>
       </c>
       <c r="B13" s="10" t="str">
         <f aca="false">IF(INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A13),$L$9:$L$38,0))&lt;=0,"",INDEX($I$9:$I$38,MATCH(LARGE($L$9:$L$38,A13),$L$9:$L$38,0)))</f>
         <v>Quality hold / inspection</v>
       </c>
-      <c r="C13" s="22" t="n">
+      <c r="C13" s="23" t="n">
         <f aca="false">IF(B13="","",INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A13),$L$9:$L$38,0)))</f>
         <v>15</v>
       </c>
@@ -24575,40 +24629,44 @@
         <f aca="false">IF(B13="","",INDEX($K$9:$K$38,MATCH(LARGE($L$9:$L$38,A13),$L$9:$L$38,0)))</f>
         <v>1</v>
       </c>
-      <c r="E13" s="23" t="n">
+      <c r="E13" s="24" t="n">
         <f aca="false">IF(OR(B13="",$B$6=0),"",C13/$B$6)</f>
         <v>0.0588235294117647</v>
       </c>
-      <c r="F13" s="23" t="n">
+      <c r="F13" s="24" t="n">
         <f aca="false">IF(OR(B13="",$B$6=0),"",SUM($C$9:C13)/$B$6)</f>
         <v>1</v>
       </c>
-      <c r="I13" s="24" t="str">
+      <c r="I13" s="25" t="str">
         <f aca="false">IF(Setup!D9="","",IF(SUMPRODUCT(--(Setup!$D$4:D8=Setup!D9))&gt;0,"",Setup!D9))</f>
         <v>Adjustment / tuning</v>
       </c>
-      <c r="J13" s="24" t="n">
+      <c r="J13" s="25" t="n">
         <f aca="false">IF(I13="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I13)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0),'Downtime Log'!$G$5:$G$1004))</f>
         <v>0</v>
       </c>
-      <c r="K13" s="24" t="n">
+      <c r="K13" s="25" t="n">
         <f aca="false">IF(I13="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I13)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>0</v>
       </c>
-      <c r="L13" s="24" t="n">
+      <c r="L13" s="25" t="n">
         <f aca="false">IF(I13="",-1,J13+(34-5)/1000000)</f>
         <v>2.9E-005</v>
       </c>
+      <c r="M13" s="26" t="n">
+        <f aca="false">IF(B13&lt;&gt;"",F13,M12)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="21" t="n">
+      <c r="A14" s="22" t="n">
         <v>6</v>
       </c>
       <c r="B14" s="10" t="str">
         <f aca="false">IF(INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A14),$L$9:$L$38,0))&lt;=0,"",INDEX($I$9:$I$38,MATCH(LARGE($L$9:$L$38,A14),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="C14" s="22" t="str">
+      <c r="C14" s="23" t="str">
         <f aca="false">IF(B14="","",INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A14),$L$9:$L$38,0)))</f>
         <v/>
       </c>
@@ -24616,40 +24674,44 @@
         <f aca="false">IF(B14="","",INDEX($K$9:$K$38,MATCH(LARGE($L$9:$L$38,A14),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="E14" s="23" t="str">
+      <c r="E14" s="24" t="str">
         <f aca="false">IF(OR(B14="",$B$6=0),"",C14/$B$6)</f>
         <v/>
       </c>
-      <c r="F14" s="23" t="str">
+      <c r="F14" s="24" t="str">
         <f aca="false">IF(OR(B14="",$B$6=0),"",SUM($C$9:C14)/$B$6)</f>
         <v/>
       </c>
-      <c r="I14" s="24" t="str">
+      <c r="I14" s="25" t="str">
         <f aca="false">IF(Setup!D10="","",IF(SUMPRODUCT(--(Setup!$D$4:D9=Setup!D10))&gt;0,"",Setup!D10))</f>
         <v>Waiting for material</v>
       </c>
-      <c r="J14" s="24" t="n">
+      <c r="J14" s="25" t="n">
         <f aca="false">IF(I14="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I14)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0),'Downtime Log'!$G$5:$G$1004))</f>
         <v>15</v>
       </c>
-      <c r="K14" s="24" t="n">
+      <c r="K14" s="25" t="n">
         <f aca="false">IF(I14="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I14)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>1</v>
       </c>
-      <c r="L14" s="24" t="n">
+      <c r="L14" s="25" t="n">
         <f aca="false">IF(I14="",-1,J14+(34-6)/1000000)</f>
         <v>15.000028</v>
       </c>
+      <c r="M14" s="26" t="n">
+        <f aca="false">IF(B14&lt;&gt;"",F14,M13)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="21" t="n">
+      <c r="A15" s="22" t="n">
         <v>7</v>
       </c>
       <c r="B15" s="10" t="str">
         <f aca="false">IF(INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A15),$L$9:$L$38,0))&lt;=0,"",INDEX($I$9:$I$38,MATCH(LARGE($L$9:$L$38,A15),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="C15" s="22" t="str">
+      <c r="C15" s="23" t="str">
         <f aca="false">IF(B15="","",INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A15),$L$9:$L$38,0)))</f>
         <v/>
       </c>
@@ -24657,40 +24719,44 @@
         <f aca="false">IF(B15="","",INDEX($K$9:$K$38,MATCH(LARGE($L$9:$L$38,A15),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="E15" s="23" t="str">
+      <c r="E15" s="24" t="str">
         <f aca="false">IF(OR(B15="",$B$6=0),"",C15/$B$6)</f>
         <v/>
       </c>
-      <c r="F15" s="23" t="str">
+      <c r="F15" s="24" t="str">
         <f aca="false">IF(OR(B15="",$B$6=0),"",SUM($C$9:C15)/$B$6)</f>
         <v/>
       </c>
-      <c r="I15" s="24" t="str">
+      <c r="I15" s="25" t="str">
         <f aca="false">IF(Setup!D11="","",IF(SUMPRODUCT(--(Setup!$D$4:D10=Setup!D11))&gt;0,"",Setup!D11))</f>
         <v>Waiting for upstream process</v>
       </c>
-      <c r="J15" s="24" t="n">
+      <c r="J15" s="25" t="n">
         <f aca="false">IF(I15="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I15)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0),'Downtime Log'!$G$5:$G$1004))</f>
         <v>0</v>
       </c>
-      <c r="K15" s="24" t="n">
+      <c r="K15" s="25" t="n">
         <f aca="false">IF(I15="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I15)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>0</v>
       </c>
-      <c r="L15" s="24" t="n">
+      <c r="L15" s="25" t="n">
         <f aca="false">IF(I15="",-1,J15+(34-7)/1000000)</f>
         <v>2.7E-005</v>
       </c>
+      <c r="M15" s="26" t="n">
+        <f aca="false">IF(B15&lt;&gt;"",F15,M14)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="21" t="n">
+      <c r="A16" s="22" t="n">
         <v>8</v>
       </c>
       <c r="B16" s="10" t="str">
         <f aca="false">IF(INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A16),$L$9:$L$38,0))&lt;=0,"",INDEX($I$9:$I$38,MATCH(LARGE($L$9:$L$38,A16),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="C16" s="22" t="str">
+      <c r="C16" s="23" t="str">
         <f aca="false">IF(B16="","",INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A16),$L$9:$L$38,0)))</f>
         <v/>
       </c>
@@ -24698,40 +24764,44 @@
         <f aca="false">IF(B16="","",INDEX($K$9:$K$38,MATCH(LARGE($L$9:$L$38,A16),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="E16" s="23" t="str">
+      <c r="E16" s="24" t="str">
         <f aca="false">IF(OR(B16="",$B$6=0),"",C16/$B$6)</f>
         <v/>
       </c>
-      <c r="F16" s="23" t="str">
+      <c r="F16" s="24" t="str">
         <f aca="false">IF(OR(B16="",$B$6=0),"",SUM($C$9:C16)/$B$6)</f>
         <v/>
       </c>
-      <c r="I16" s="24" t="str">
+      <c r="I16" s="25" t="str">
         <f aca="false">IF(Setup!D12="","",IF(SUMPRODUCT(--(Setup!$D$4:D11=Setup!D12))&gt;0,"",Setup!D12))</f>
         <v>Quality hold / inspection</v>
       </c>
-      <c r="J16" s="24" t="n">
+      <c r="J16" s="25" t="n">
         <f aca="false">IF(I16="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I16)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0),'Downtime Log'!$G$5:$G$1004))</f>
         <v>15</v>
       </c>
-      <c r="K16" s="24" t="n">
+      <c r="K16" s="25" t="n">
         <f aca="false">IF(I16="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I16)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>1</v>
       </c>
-      <c r="L16" s="24" t="n">
+      <c r="L16" s="25" t="n">
         <f aca="false">IF(I16="",-1,J16+(34-8)/1000000)</f>
         <v>15.000026</v>
       </c>
+      <c r="M16" s="26" t="n">
+        <f aca="false">IF(B16&lt;&gt;"",F16,M15)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="21" t="n">
+      <c r="A17" s="22" t="n">
         <v>9</v>
       </c>
       <c r="B17" s="10" t="str">
         <f aca="false">IF(INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A17),$L$9:$L$38,0))&lt;=0,"",INDEX($I$9:$I$38,MATCH(LARGE($L$9:$L$38,A17),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="C17" s="22" t="str">
+      <c r="C17" s="23" t="str">
         <f aca="false">IF(B17="","",INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A17),$L$9:$L$38,0)))</f>
         <v/>
       </c>
@@ -24739,40 +24809,44 @@
         <f aca="false">IF(B17="","",INDEX($K$9:$K$38,MATCH(LARGE($L$9:$L$38,A17),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="E17" s="23" t="str">
+      <c r="E17" s="24" t="str">
         <f aca="false">IF(OR(B17="",$B$6=0),"",C17/$B$6)</f>
         <v/>
       </c>
-      <c r="F17" s="23" t="str">
+      <c r="F17" s="24" t="str">
         <f aca="false">IF(OR(B17="",$B$6=0),"",SUM($C$9:C17)/$B$6)</f>
         <v/>
       </c>
-      <c r="I17" s="24" t="str">
+      <c r="I17" s="25" t="str">
         <f aca="false">IF(Setup!D13="","",IF(SUMPRODUCT(--(Setup!$D$4:D12=Setup!D13))&gt;0,"",Setup!D13))</f>
         <v>No operator available</v>
       </c>
-      <c r="J17" s="24" t="n">
+      <c r="J17" s="25" t="n">
         <f aca="false">IF(I17="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I17)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0),'Downtime Log'!$G$5:$G$1004))</f>
         <v>0</v>
       </c>
-      <c r="K17" s="24" t="n">
+      <c r="K17" s="25" t="n">
         <f aca="false">IF(I17="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I17)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>0</v>
       </c>
-      <c r="L17" s="24" t="n">
+      <c r="L17" s="25" t="n">
         <f aca="false">IF(I17="",-1,J17+(34-9)/1000000)</f>
         <v>2.5E-005</v>
       </c>
+      <c r="M17" s="26" t="n">
+        <f aca="false">IF(B17&lt;&gt;"",F17,M16)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="21" t="n">
+      <c r="A18" s="22" t="n">
         <v>10</v>
       </c>
       <c r="B18" s="10" t="str">
         <f aca="false">IF(INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A18),$L$9:$L$38,0))&lt;=0,"",INDEX($I$9:$I$38,MATCH(LARGE($L$9:$L$38,A18),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="C18" s="22" t="str">
+      <c r="C18" s="23" t="str">
         <f aca="false">IF(B18="","",INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A18),$L$9:$L$38,0)))</f>
         <v/>
       </c>
@@ -24780,40 +24854,44 @@
         <f aca="false">IF(B18="","",INDEX($K$9:$K$38,MATCH(LARGE($L$9:$L$38,A18),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="E18" s="23" t="str">
+      <c r="E18" s="24" t="str">
         <f aca="false">IF(OR(B18="",$B$6=0),"",C18/$B$6)</f>
         <v/>
       </c>
-      <c r="F18" s="23" t="str">
+      <c r="F18" s="24" t="str">
         <f aca="false">IF(OR(B18="",$B$6=0),"",SUM($C$9:C18)/$B$6)</f>
         <v/>
       </c>
-      <c r="I18" s="24" t="str">
+      <c r="I18" s="25" t="str">
         <f aca="false">IF(Setup!D14="","",IF(SUMPRODUCT(--(Setup!$D$4:D13=Setup!D14))&gt;0,"",Setup!D14))</f>
         <v>Planned maintenance</v>
       </c>
-      <c r="J18" s="24" t="n">
+      <c r="J18" s="25" t="n">
         <f aca="false">IF(I18="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I18)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0),'Downtime Log'!$G$5:$G$1004))</f>
         <v>0</v>
       </c>
-      <c r="K18" s="24" t="n">
+      <c r="K18" s="25" t="n">
         <f aca="false">IF(I18="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I18)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>0</v>
       </c>
-      <c r="L18" s="24" t="n">
+      <c r="L18" s="25" t="n">
         <f aca="false">IF(I18="",-1,J18+(34-10)/1000000)</f>
         <v>2.4E-005</v>
       </c>
+      <c r="M18" s="26" t="n">
+        <f aca="false">IF(B18&lt;&gt;"",F18,M17)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="21" t="n">
+      <c r="A19" s="22" t="n">
         <v>11</v>
       </c>
       <c r="B19" s="10" t="str">
         <f aca="false">IF(INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A19),$L$9:$L$38,0))&lt;=0,"",INDEX($I$9:$I$38,MATCH(LARGE($L$9:$L$38,A19),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="C19" s="22" t="str">
+      <c r="C19" s="23" t="str">
         <f aca="false">IF(B19="","",INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A19),$L$9:$L$38,0)))</f>
         <v/>
       </c>
@@ -24821,40 +24899,44 @@
         <f aca="false">IF(B19="","",INDEX($K$9:$K$38,MATCH(LARGE($L$9:$L$38,A19),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="E19" s="23" t="str">
+      <c r="E19" s="24" t="str">
         <f aca="false">IF(OR(B19="",$B$6=0),"",C19/$B$6)</f>
         <v/>
       </c>
-      <c r="F19" s="23" t="str">
+      <c r="F19" s="24" t="str">
         <f aca="false">IF(OR(B19="",$B$6=0),"",SUM($C$9:C19)/$B$6)</f>
         <v/>
       </c>
-      <c r="I19" s="24" t="str">
+      <c r="I19" s="25" t="str">
         <f aca="false">IF(Setup!D15="","",IF(SUMPRODUCT(--(Setup!$D$4:D14=Setup!D15))&gt;0,"",Setup!D15))</f>
         <v>Meeting / training</v>
       </c>
-      <c r="J19" s="24" t="n">
+      <c r="J19" s="25" t="n">
         <f aca="false">IF(I19="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I19)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0),'Downtime Log'!$G$5:$G$1004))</f>
         <v>0</v>
       </c>
-      <c r="K19" s="24" t="n">
+      <c r="K19" s="25" t="n">
         <f aca="false">IF(I19="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I19)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>0</v>
       </c>
-      <c r="L19" s="24" t="n">
+      <c r="L19" s="25" t="n">
         <f aca="false">IF(I19="",-1,J19+(34-11)/1000000)</f>
         <v>2.3E-005</v>
       </c>
+      <c r="M19" s="26" t="n">
+        <f aca="false">IF(B19&lt;&gt;"",F19,M18)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="21" t="n">
+      <c r="A20" s="22" t="n">
         <v>12</v>
       </c>
       <c r="B20" s="10" t="str">
         <f aca="false">IF(INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A20),$L$9:$L$38,0))&lt;=0,"",INDEX($I$9:$I$38,MATCH(LARGE($L$9:$L$38,A20),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="C20" s="22" t="str">
+      <c r="C20" s="23" t="str">
         <f aca="false">IF(B20="","",INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A20),$L$9:$L$38,0)))</f>
         <v/>
       </c>
@@ -24862,40 +24944,44 @@
         <f aca="false">IF(B20="","",INDEX($K$9:$K$38,MATCH(LARGE($L$9:$L$38,A20),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="E20" s="23" t="str">
+      <c r="E20" s="24" t="str">
         <f aca="false">IF(OR(B20="",$B$6=0),"",C20/$B$6)</f>
         <v/>
       </c>
-      <c r="F20" s="23" t="str">
+      <c r="F20" s="24" t="str">
         <f aca="false">IF(OR(B20="",$B$6=0),"",SUM($C$9:C20)/$B$6)</f>
         <v/>
       </c>
-      <c r="I20" s="24" t="str">
+      <c r="I20" s="25" t="str">
         <f aca="false">IF(Setup!D16="","",IF(SUMPRODUCT(--(Setup!$D$4:D15=Setup!D16))&gt;0,"",Setup!D16))</f>
         <v>Other (describe in notes)</v>
       </c>
-      <c r="J20" s="24" t="n">
+      <c r="J20" s="25" t="n">
         <f aca="false">IF(I20="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I20)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0),'Downtime Log'!$G$5:$G$1004))</f>
         <v>0</v>
       </c>
-      <c r="K20" s="24" t="n">
+      <c r="K20" s="25" t="n">
         <f aca="false">IF(I20="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I20)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>0</v>
       </c>
-      <c r="L20" s="24" t="n">
+      <c r="L20" s="25" t="n">
         <f aca="false">IF(I20="",-1,J20+(34-12)/1000000)</f>
         <v>2.2E-005</v>
       </c>
+      <c r="M20" s="26" t="n">
+        <f aca="false">IF(B20&lt;&gt;"",F20,M19)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="21" t="n">
+      <c r="A21" s="22" t="n">
         <v>13</v>
       </c>
       <c r="B21" s="10" t="str">
         <f aca="false">IF(INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A21),$L$9:$L$38,0))&lt;=0,"",INDEX($I$9:$I$38,MATCH(LARGE($L$9:$L$38,A21),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="C21" s="22" t="str">
+      <c r="C21" s="23" t="str">
         <f aca="false">IF(B21="","",INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A21),$L$9:$L$38,0)))</f>
         <v/>
       </c>
@@ -24903,40 +24989,44 @@
         <f aca="false">IF(B21="","",INDEX($K$9:$K$38,MATCH(LARGE($L$9:$L$38,A21),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="E21" s="23" t="str">
+      <c r="E21" s="24" t="str">
         <f aca="false">IF(OR(B21="",$B$6=0),"",C21/$B$6)</f>
         <v/>
       </c>
-      <c r="F21" s="23" t="str">
+      <c r="F21" s="24" t="str">
         <f aca="false">IF(OR(B21="",$B$6=0),"",SUM($C$9:C21)/$B$6)</f>
         <v/>
       </c>
-      <c r="I21" s="24" t="str">
+      <c r="I21" s="25" t="str">
         <f aca="false">IF(Setup!D17="","",IF(SUMPRODUCT(--(Setup!$D$4:D16=Setup!D17))&gt;0,"",Setup!D17))</f>
         <v/>
       </c>
-      <c r="J21" s="24" t="n">
+      <c r="J21" s="25" t="n">
         <f aca="false">IF(I21="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I21)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0),'Downtime Log'!$G$5:$G$1004))</f>
         <v>0</v>
       </c>
-      <c r="K21" s="24" t="n">
+      <c r="K21" s="25" t="n">
         <f aca="false">IF(I21="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I21)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>0</v>
       </c>
-      <c r="L21" s="24" t="n">
+      <c r="L21" s="25" t="n">
         <f aca="false">IF(I21="",-1,J21+(34-13)/1000000)</f>
         <v>-1</v>
       </c>
+      <c r="M21" s="26" t="n">
+        <f aca="false">IF(B21&lt;&gt;"",F21,M20)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="21" t="n">
+      <c r="A22" s="22" t="n">
         <v>14</v>
       </c>
       <c r="B22" s="10" t="str">
         <f aca="false">IF(INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A22),$L$9:$L$38,0))&lt;=0,"",INDEX($I$9:$I$38,MATCH(LARGE($L$9:$L$38,A22),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="C22" s="22" t="str">
+      <c r="C22" s="23" t="str">
         <f aca="false">IF(B22="","",INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A22),$L$9:$L$38,0)))</f>
         <v/>
       </c>
@@ -24944,40 +25034,44 @@
         <f aca="false">IF(B22="","",INDEX($K$9:$K$38,MATCH(LARGE($L$9:$L$38,A22),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="E22" s="23" t="str">
+      <c r="E22" s="24" t="str">
         <f aca="false">IF(OR(B22="",$B$6=0),"",C22/$B$6)</f>
         <v/>
       </c>
-      <c r="F22" s="23" t="str">
+      <c r="F22" s="24" t="str">
         <f aca="false">IF(OR(B22="",$B$6=0),"",SUM($C$9:C22)/$B$6)</f>
         <v/>
       </c>
-      <c r="I22" s="24" t="str">
+      <c r="I22" s="25" t="str">
         <f aca="false">IF(Setup!D18="","",IF(SUMPRODUCT(--(Setup!$D$4:D17=Setup!D18))&gt;0,"",Setup!D18))</f>
         <v/>
       </c>
-      <c r="J22" s="24" t="n">
+      <c r="J22" s="25" t="n">
         <f aca="false">IF(I22="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I22)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0),'Downtime Log'!$G$5:$G$1004))</f>
         <v>0</v>
       </c>
-      <c r="K22" s="24" t="n">
+      <c r="K22" s="25" t="n">
         <f aca="false">IF(I22="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I22)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>0</v>
       </c>
-      <c r="L22" s="24" t="n">
+      <c r="L22" s="25" t="n">
         <f aca="false">IF(I22="",-1,J22+(34-14)/1000000)</f>
         <v>-1</v>
       </c>
+      <c r="M22" s="26" t="n">
+        <f aca="false">IF(B22&lt;&gt;"",F22,M21)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="21" t="n">
+      <c r="A23" s="22" t="n">
         <v>15</v>
       </c>
       <c r="B23" s="10" t="str">
         <f aca="false">IF(INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A23),$L$9:$L$38,0))&lt;=0,"",INDEX($I$9:$I$38,MATCH(LARGE($L$9:$L$38,A23),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="C23" s="22" t="str">
+      <c r="C23" s="23" t="str">
         <f aca="false">IF(B23="","",INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A23),$L$9:$L$38,0)))</f>
         <v/>
       </c>
@@ -24985,40 +25079,44 @@
         <f aca="false">IF(B23="","",INDEX($K$9:$K$38,MATCH(LARGE($L$9:$L$38,A23),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="E23" s="23" t="str">
+      <c r="E23" s="24" t="str">
         <f aca="false">IF(OR(B23="",$B$6=0),"",C23/$B$6)</f>
         <v/>
       </c>
-      <c r="F23" s="23" t="str">
+      <c r="F23" s="24" t="str">
         <f aca="false">IF(OR(B23="",$B$6=0),"",SUM($C$9:C23)/$B$6)</f>
         <v/>
       </c>
-      <c r="I23" s="24" t="str">
+      <c r="I23" s="25" t="str">
         <f aca="false">IF(Setup!D19="","",IF(SUMPRODUCT(--(Setup!$D$4:D18=Setup!D19))&gt;0,"",Setup!D19))</f>
         <v/>
       </c>
-      <c r="J23" s="24" t="n">
+      <c r="J23" s="25" t="n">
         <f aca="false">IF(I23="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I23)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0),'Downtime Log'!$G$5:$G$1004))</f>
         <v>0</v>
       </c>
-      <c r="K23" s="24" t="n">
+      <c r="K23" s="25" t="n">
         <f aca="false">IF(I23="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I23)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>0</v>
       </c>
-      <c r="L23" s="24" t="n">
+      <c r="L23" s="25" t="n">
         <f aca="false">IF(I23="",-1,J23+(34-15)/1000000)</f>
         <v>-1</v>
       </c>
+      <c r="M23" s="26" t="n">
+        <f aca="false">IF(B23&lt;&gt;"",F23,M22)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="21" t="n">
+      <c r="A24" s="22" t="n">
         <v>16</v>
       </c>
       <c r="B24" s="10" t="str">
         <f aca="false">IF(INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A24),$L$9:$L$38,0))&lt;=0,"",INDEX($I$9:$I$38,MATCH(LARGE($L$9:$L$38,A24),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="C24" s="22" t="str">
+      <c r="C24" s="23" t="str">
         <f aca="false">IF(B24="","",INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A24),$L$9:$L$38,0)))</f>
         <v/>
       </c>
@@ -25026,40 +25124,44 @@
         <f aca="false">IF(B24="","",INDEX($K$9:$K$38,MATCH(LARGE($L$9:$L$38,A24),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="E24" s="23" t="str">
+      <c r="E24" s="24" t="str">
         <f aca="false">IF(OR(B24="",$B$6=0),"",C24/$B$6)</f>
         <v/>
       </c>
-      <c r="F24" s="23" t="str">
+      <c r="F24" s="24" t="str">
         <f aca="false">IF(OR(B24="",$B$6=0),"",SUM($C$9:C24)/$B$6)</f>
         <v/>
       </c>
-      <c r="I24" s="24" t="str">
+      <c r="I24" s="25" t="str">
         <f aca="false">IF(Setup!D20="","",IF(SUMPRODUCT(--(Setup!$D$4:D19=Setup!D20))&gt;0,"",Setup!D20))</f>
         <v/>
       </c>
-      <c r="J24" s="24" t="n">
+      <c r="J24" s="25" t="n">
         <f aca="false">IF(I24="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I24)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0),'Downtime Log'!$G$5:$G$1004))</f>
         <v>0</v>
       </c>
-      <c r="K24" s="24" t="n">
+      <c r="K24" s="25" t="n">
         <f aca="false">IF(I24="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I24)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>0</v>
       </c>
-      <c r="L24" s="24" t="n">
+      <c r="L24" s="25" t="n">
         <f aca="false">IF(I24="",-1,J24+(34-16)/1000000)</f>
         <v>-1</v>
       </c>
+      <c r="M24" s="26" t="n">
+        <f aca="false">IF(B24&lt;&gt;"",F24,M23)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="21" t="n">
+      <c r="A25" s="22" t="n">
         <v>17</v>
       </c>
       <c r="B25" s="10" t="str">
         <f aca="false">IF(INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A25),$L$9:$L$38,0))&lt;=0,"",INDEX($I$9:$I$38,MATCH(LARGE($L$9:$L$38,A25),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="C25" s="22" t="str">
+      <c r="C25" s="23" t="str">
         <f aca="false">IF(B25="","",INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A25),$L$9:$L$38,0)))</f>
         <v/>
       </c>
@@ -25067,40 +25169,44 @@
         <f aca="false">IF(B25="","",INDEX($K$9:$K$38,MATCH(LARGE($L$9:$L$38,A25),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="E25" s="23" t="str">
+      <c r="E25" s="24" t="str">
         <f aca="false">IF(OR(B25="",$B$6=0),"",C25/$B$6)</f>
         <v/>
       </c>
-      <c r="F25" s="23" t="str">
+      <c r="F25" s="24" t="str">
         <f aca="false">IF(OR(B25="",$B$6=0),"",SUM($C$9:C25)/$B$6)</f>
         <v/>
       </c>
-      <c r="I25" s="24" t="str">
+      <c r="I25" s="25" t="str">
         <f aca="false">IF(Setup!D21="","",IF(SUMPRODUCT(--(Setup!$D$4:D20=Setup!D21))&gt;0,"",Setup!D21))</f>
         <v/>
       </c>
-      <c r="J25" s="24" t="n">
+      <c r="J25" s="25" t="n">
         <f aca="false">IF(I25="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I25)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0),'Downtime Log'!$G$5:$G$1004))</f>
         <v>0</v>
       </c>
-      <c r="K25" s="24" t="n">
+      <c r="K25" s="25" t="n">
         <f aca="false">IF(I25="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I25)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>0</v>
       </c>
-      <c r="L25" s="24" t="n">
+      <c r="L25" s="25" t="n">
         <f aca="false">IF(I25="",-1,J25+(34-17)/1000000)</f>
         <v>-1</v>
       </c>
+      <c r="M25" s="26" t="n">
+        <f aca="false">IF(B25&lt;&gt;"",F25,M24)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="21" t="n">
+      <c r="A26" s="22" t="n">
         <v>18</v>
       </c>
       <c r="B26" s="10" t="str">
         <f aca="false">IF(INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A26),$L$9:$L$38,0))&lt;=0,"",INDEX($I$9:$I$38,MATCH(LARGE($L$9:$L$38,A26),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="C26" s="22" t="str">
+      <c r="C26" s="23" t="str">
         <f aca="false">IF(B26="","",INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A26),$L$9:$L$38,0)))</f>
         <v/>
       </c>
@@ -25108,40 +25214,44 @@
         <f aca="false">IF(B26="","",INDEX($K$9:$K$38,MATCH(LARGE($L$9:$L$38,A26),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="E26" s="23" t="str">
+      <c r="E26" s="24" t="str">
         <f aca="false">IF(OR(B26="",$B$6=0),"",C26/$B$6)</f>
         <v/>
       </c>
-      <c r="F26" s="23" t="str">
+      <c r="F26" s="24" t="str">
         <f aca="false">IF(OR(B26="",$B$6=0),"",SUM($C$9:C26)/$B$6)</f>
         <v/>
       </c>
-      <c r="I26" s="24" t="str">
+      <c r="I26" s="25" t="str">
         <f aca="false">IF(Setup!D22="","",IF(SUMPRODUCT(--(Setup!$D$4:D21=Setup!D22))&gt;0,"",Setup!D22))</f>
         <v/>
       </c>
-      <c r="J26" s="24" t="n">
+      <c r="J26" s="25" t="n">
         <f aca="false">IF(I26="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I26)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0),'Downtime Log'!$G$5:$G$1004))</f>
         <v>0</v>
       </c>
-      <c r="K26" s="24" t="n">
+      <c r="K26" s="25" t="n">
         <f aca="false">IF(I26="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I26)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>0</v>
       </c>
-      <c r="L26" s="24" t="n">
+      <c r="L26" s="25" t="n">
         <f aca="false">IF(I26="",-1,J26+(34-18)/1000000)</f>
         <v>-1</v>
       </c>
+      <c r="M26" s="26" t="n">
+        <f aca="false">IF(B26&lt;&gt;"",F26,M25)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="21" t="n">
+      <c r="A27" s="22" t="n">
         <v>19</v>
       </c>
       <c r="B27" s="10" t="str">
         <f aca="false">IF(INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A27),$L$9:$L$38,0))&lt;=0,"",INDEX($I$9:$I$38,MATCH(LARGE($L$9:$L$38,A27),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="C27" s="22" t="str">
+      <c r="C27" s="23" t="str">
         <f aca="false">IF(B27="","",INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A27),$L$9:$L$38,0)))</f>
         <v/>
       </c>
@@ -25149,40 +25259,44 @@
         <f aca="false">IF(B27="","",INDEX($K$9:$K$38,MATCH(LARGE($L$9:$L$38,A27),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="E27" s="23" t="str">
+      <c r="E27" s="24" t="str">
         <f aca="false">IF(OR(B27="",$B$6=0),"",C27/$B$6)</f>
         <v/>
       </c>
-      <c r="F27" s="23" t="str">
+      <c r="F27" s="24" t="str">
         <f aca="false">IF(OR(B27="",$B$6=0),"",SUM($C$9:C27)/$B$6)</f>
         <v/>
       </c>
-      <c r="I27" s="24" t="str">
+      <c r="I27" s="25" t="str">
         <f aca="false">IF(Setup!D23="","",IF(SUMPRODUCT(--(Setup!$D$4:D22=Setup!D23))&gt;0,"",Setup!D23))</f>
         <v/>
       </c>
-      <c r="J27" s="24" t="n">
+      <c r="J27" s="25" t="n">
         <f aca="false">IF(I27="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I27)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0),'Downtime Log'!$G$5:$G$1004))</f>
         <v>0</v>
       </c>
-      <c r="K27" s="24" t="n">
+      <c r="K27" s="25" t="n">
         <f aca="false">IF(I27="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I27)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>0</v>
       </c>
-      <c r="L27" s="24" t="n">
+      <c r="L27" s="25" t="n">
         <f aca="false">IF(I27="",-1,J27+(34-19)/1000000)</f>
         <v>-1</v>
       </c>
+      <c r="M27" s="26" t="n">
+        <f aca="false">IF(B27&lt;&gt;"",F27,M26)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="21" t="n">
+      <c r="A28" s="22" t="n">
         <v>20</v>
       </c>
       <c r="B28" s="10" t="str">
         <f aca="false">IF(INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A28),$L$9:$L$38,0))&lt;=0,"",INDEX($I$9:$I$38,MATCH(LARGE($L$9:$L$38,A28),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="C28" s="22" t="str">
+      <c r="C28" s="23" t="str">
         <f aca="false">IF(B28="","",INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A28),$L$9:$L$38,0)))</f>
         <v/>
       </c>
@@ -25190,40 +25304,44 @@
         <f aca="false">IF(B28="","",INDEX($K$9:$K$38,MATCH(LARGE($L$9:$L$38,A28),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="E28" s="23" t="str">
+      <c r="E28" s="24" t="str">
         <f aca="false">IF(OR(B28="",$B$6=0),"",C28/$B$6)</f>
         <v/>
       </c>
-      <c r="F28" s="23" t="str">
+      <c r="F28" s="24" t="str">
         <f aca="false">IF(OR(B28="",$B$6=0),"",SUM($C$9:C28)/$B$6)</f>
         <v/>
       </c>
-      <c r="I28" s="24" t="str">
+      <c r="I28" s="25" t="str">
         <f aca="false">IF(Setup!D24="","",IF(SUMPRODUCT(--(Setup!$D$4:D23=Setup!D24))&gt;0,"",Setup!D24))</f>
         <v/>
       </c>
-      <c r="J28" s="24" t="n">
+      <c r="J28" s="25" t="n">
         <f aca="false">IF(I28="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I28)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0),'Downtime Log'!$G$5:$G$1004))</f>
         <v>0</v>
       </c>
-      <c r="K28" s="24" t="n">
+      <c r="K28" s="25" t="n">
         <f aca="false">IF(I28="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I28)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>0</v>
       </c>
-      <c r="L28" s="24" t="n">
+      <c r="L28" s="25" t="n">
         <f aca="false">IF(I28="",-1,J28+(34-20)/1000000)</f>
         <v>-1</v>
       </c>
+      <c r="M28" s="26" t="n">
+        <f aca="false">IF(B28&lt;&gt;"",F28,M27)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="21" t="n">
+      <c r="A29" s="22" t="n">
         <v>21</v>
       </c>
       <c r="B29" s="10" t="str">
         <f aca="false">IF(INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A29),$L$9:$L$38,0))&lt;=0,"",INDEX($I$9:$I$38,MATCH(LARGE($L$9:$L$38,A29),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="C29" s="22" t="str">
+      <c r="C29" s="23" t="str">
         <f aca="false">IF(B29="","",INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A29),$L$9:$L$38,0)))</f>
         <v/>
       </c>
@@ -25231,40 +25349,44 @@
         <f aca="false">IF(B29="","",INDEX($K$9:$K$38,MATCH(LARGE($L$9:$L$38,A29),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="E29" s="23" t="str">
+      <c r="E29" s="24" t="str">
         <f aca="false">IF(OR(B29="",$B$6=0),"",C29/$B$6)</f>
         <v/>
       </c>
-      <c r="F29" s="23" t="str">
+      <c r="F29" s="24" t="str">
         <f aca="false">IF(OR(B29="",$B$6=0),"",SUM($C$9:C29)/$B$6)</f>
         <v/>
       </c>
-      <c r="I29" s="24" t="str">
+      <c r="I29" s="25" t="str">
         <f aca="false">IF(Setup!D25="","",IF(SUMPRODUCT(--(Setup!$D$4:D24=Setup!D25))&gt;0,"",Setup!D25))</f>
         <v/>
       </c>
-      <c r="J29" s="24" t="n">
+      <c r="J29" s="25" t="n">
         <f aca="false">IF(I29="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I29)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0),'Downtime Log'!$G$5:$G$1004))</f>
         <v>0</v>
       </c>
-      <c r="K29" s="24" t="n">
+      <c r="K29" s="25" t="n">
         <f aca="false">IF(I29="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I29)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>0</v>
       </c>
-      <c r="L29" s="24" t="n">
+      <c r="L29" s="25" t="n">
         <f aca="false">IF(I29="",-1,J29+(34-21)/1000000)</f>
         <v>-1</v>
       </c>
+      <c r="M29" s="26" t="n">
+        <f aca="false">IF(B29&lt;&gt;"",F29,M28)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="21" t="n">
+      <c r="A30" s="22" t="n">
         <v>22</v>
       </c>
       <c r="B30" s="10" t="str">
         <f aca="false">IF(INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A30),$L$9:$L$38,0))&lt;=0,"",INDEX($I$9:$I$38,MATCH(LARGE($L$9:$L$38,A30),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="C30" s="22" t="str">
+      <c r="C30" s="23" t="str">
         <f aca="false">IF(B30="","",INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A30),$L$9:$L$38,0)))</f>
         <v/>
       </c>
@@ -25272,40 +25394,44 @@
         <f aca="false">IF(B30="","",INDEX($K$9:$K$38,MATCH(LARGE($L$9:$L$38,A30),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="E30" s="23" t="str">
+      <c r="E30" s="24" t="str">
         <f aca="false">IF(OR(B30="",$B$6=0),"",C30/$B$6)</f>
         <v/>
       </c>
-      <c r="F30" s="23" t="str">
+      <c r="F30" s="24" t="str">
         <f aca="false">IF(OR(B30="",$B$6=0),"",SUM($C$9:C30)/$B$6)</f>
         <v/>
       </c>
-      <c r="I30" s="24" t="str">
+      <c r="I30" s="25" t="str">
         <f aca="false">IF(Setup!D26="","",IF(SUMPRODUCT(--(Setup!$D$4:D25=Setup!D26))&gt;0,"",Setup!D26))</f>
         <v/>
       </c>
-      <c r="J30" s="24" t="n">
+      <c r="J30" s="25" t="n">
         <f aca="false">IF(I30="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I30)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0),'Downtime Log'!$G$5:$G$1004))</f>
         <v>0</v>
       </c>
-      <c r="K30" s="24" t="n">
+      <c r="K30" s="25" t="n">
         <f aca="false">IF(I30="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I30)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>0</v>
       </c>
-      <c r="L30" s="24" t="n">
+      <c r="L30" s="25" t="n">
         <f aca="false">IF(I30="",-1,J30+(34-22)/1000000)</f>
         <v>-1</v>
       </c>
+      <c r="M30" s="26" t="n">
+        <f aca="false">IF(B30&lt;&gt;"",F30,M29)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="21" t="n">
+      <c r="A31" s="22" t="n">
         <v>23</v>
       </c>
       <c r="B31" s="10" t="str">
         <f aca="false">IF(INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A31),$L$9:$L$38,0))&lt;=0,"",INDEX($I$9:$I$38,MATCH(LARGE($L$9:$L$38,A31),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="C31" s="22" t="str">
+      <c r="C31" s="23" t="str">
         <f aca="false">IF(B31="","",INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A31),$L$9:$L$38,0)))</f>
         <v/>
       </c>
@@ -25313,40 +25439,44 @@
         <f aca="false">IF(B31="","",INDEX($K$9:$K$38,MATCH(LARGE($L$9:$L$38,A31),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="E31" s="23" t="str">
+      <c r="E31" s="24" t="str">
         <f aca="false">IF(OR(B31="",$B$6=0),"",C31/$B$6)</f>
         <v/>
       </c>
-      <c r="F31" s="23" t="str">
+      <c r="F31" s="24" t="str">
         <f aca="false">IF(OR(B31="",$B$6=0),"",SUM($C$9:C31)/$B$6)</f>
         <v/>
       </c>
-      <c r="I31" s="24" t="str">
+      <c r="I31" s="25" t="str">
         <f aca="false">IF(Setup!D27="","",IF(SUMPRODUCT(--(Setup!$D$4:D26=Setup!D27))&gt;0,"",Setup!D27))</f>
         <v/>
       </c>
-      <c r="J31" s="24" t="n">
+      <c r="J31" s="25" t="n">
         <f aca="false">IF(I31="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I31)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0),'Downtime Log'!$G$5:$G$1004))</f>
         <v>0</v>
       </c>
-      <c r="K31" s="24" t="n">
+      <c r="K31" s="25" t="n">
         <f aca="false">IF(I31="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I31)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>0</v>
       </c>
-      <c r="L31" s="24" t="n">
+      <c r="L31" s="25" t="n">
         <f aca="false">IF(I31="",-1,J31+(34-23)/1000000)</f>
         <v>-1</v>
       </c>
+      <c r="M31" s="26" t="n">
+        <f aca="false">IF(B31&lt;&gt;"",F31,M30)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="21" t="n">
+      <c r="A32" s="22" t="n">
         <v>24</v>
       </c>
       <c r="B32" s="10" t="str">
         <f aca="false">IF(INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A32),$L$9:$L$38,0))&lt;=0,"",INDEX($I$9:$I$38,MATCH(LARGE($L$9:$L$38,A32),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="C32" s="22" t="str">
+      <c r="C32" s="23" t="str">
         <f aca="false">IF(B32="","",INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A32),$L$9:$L$38,0)))</f>
         <v/>
       </c>
@@ -25354,40 +25484,44 @@
         <f aca="false">IF(B32="","",INDEX($K$9:$K$38,MATCH(LARGE($L$9:$L$38,A32),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="E32" s="23" t="str">
+      <c r="E32" s="24" t="str">
         <f aca="false">IF(OR(B32="",$B$6=0),"",C32/$B$6)</f>
         <v/>
       </c>
-      <c r="F32" s="23" t="str">
+      <c r="F32" s="24" t="str">
         <f aca="false">IF(OR(B32="",$B$6=0),"",SUM($C$9:C32)/$B$6)</f>
         <v/>
       </c>
-      <c r="I32" s="24" t="str">
+      <c r="I32" s="25" t="str">
         <f aca="false">IF(Setup!D28="","",IF(SUMPRODUCT(--(Setup!$D$4:D27=Setup!D28))&gt;0,"",Setup!D28))</f>
         <v/>
       </c>
-      <c r="J32" s="24" t="n">
+      <c r="J32" s="25" t="n">
         <f aca="false">IF(I32="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I32)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0),'Downtime Log'!$G$5:$G$1004))</f>
         <v>0</v>
       </c>
-      <c r="K32" s="24" t="n">
+      <c r="K32" s="25" t="n">
         <f aca="false">IF(I32="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I32)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>0</v>
       </c>
-      <c r="L32" s="24" t="n">
+      <c r="L32" s="25" t="n">
         <f aca="false">IF(I32="",-1,J32+(34-24)/1000000)</f>
         <v>-1</v>
       </c>
+      <c r="M32" s="26" t="n">
+        <f aca="false">IF(B32&lt;&gt;"",F32,M31)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="21" t="n">
+      <c r="A33" s="22" t="n">
         <v>25</v>
       </c>
       <c r="B33" s="10" t="str">
         <f aca="false">IF(INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A33),$L$9:$L$38,0))&lt;=0,"",INDEX($I$9:$I$38,MATCH(LARGE($L$9:$L$38,A33),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="C33" s="22" t="str">
+      <c r="C33" s="23" t="str">
         <f aca="false">IF(B33="","",INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A33),$L$9:$L$38,0)))</f>
         <v/>
       </c>
@@ -25395,40 +25529,44 @@
         <f aca="false">IF(B33="","",INDEX($K$9:$K$38,MATCH(LARGE($L$9:$L$38,A33),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="E33" s="23" t="str">
+      <c r="E33" s="24" t="str">
         <f aca="false">IF(OR(B33="",$B$6=0),"",C33/$B$6)</f>
         <v/>
       </c>
-      <c r="F33" s="23" t="str">
+      <c r="F33" s="24" t="str">
         <f aca="false">IF(OR(B33="",$B$6=0),"",SUM($C$9:C33)/$B$6)</f>
         <v/>
       </c>
-      <c r="I33" s="24" t="str">
+      <c r="I33" s="25" t="str">
         <f aca="false">IF(Setup!D29="","",IF(SUMPRODUCT(--(Setup!$D$4:D28=Setup!D29))&gt;0,"",Setup!D29))</f>
         <v/>
       </c>
-      <c r="J33" s="24" t="n">
+      <c r="J33" s="25" t="n">
         <f aca="false">IF(I33="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I33)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0),'Downtime Log'!$G$5:$G$1004))</f>
         <v>0</v>
       </c>
-      <c r="K33" s="24" t="n">
+      <c r="K33" s="25" t="n">
         <f aca="false">IF(I33="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I33)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>0</v>
       </c>
-      <c r="L33" s="24" t="n">
+      <c r="L33" s="25" t="n">
         <f aca="false">IF(I33="",-1,J33+(34-25)/1000000)</f>
         <v>-1</v>
       </c>
+      <c r="M33" s="26" t="n">
+        <f aca="false">IF(B33&lt;&gt;"",F33,M32)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="21" t="n">
+      <c r="A34" s="22" t="n">
         <v>26</v>
       </c>
       <c r="B34" s="10" t="str">
         <f aca="false">IF(INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A34),$L$9:$L$38,0))&lt;=0,"",INDEX($I$9:$I$38,MATCH(LARGE($L$9:$L$38,A34),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="C34" s="22" t="str">
+      <c r="C34" s="23" t="str">
         <f aca="false">IF(B34="","",INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A34),$L$9:$L$38,0)))</f>
         <v/>
       </c>
@@ -25436,40 +25574,44 @@
         <f aca="false">IF(B34="","",INDEX($K$9:$K$38,MATCH(LARGE($L$9:$L$38,A34),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="E34" s="23" t="str">
+      <c r="E34" s="24" t="str">
         <f aca="false">IF(OR(B34="",$B$6=0),"",C34/$B$6)</f>
         <v/>
       </c>
-      <c r="F34" s="23" t="str">
+      <c r="F34" s="24" t="str">
         <f aca="false">IF(OR(B34="",$B$6=0),"",SUM($C$9:C34)/$B$6)</f>
         <v/>
       </c>
-      <c r="I34" s="24" t="str">
+      <c r="I34" s="25" t="str">
         <f aca="false">IF(Setup!D30="","",IF(SUMPRODUCT(--(Setup!$D$4:D29=Setup!D30))&gt;0,"",Setup!D30))</f>
         <v/>
       </c>
-      <c r="J34" s="24" t="n">
+      <c r="J34" s="25" t="n">
         <f aca="false">IF(I34="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I34)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0),'Downtime Log'!$G$5:$G$1004))</f>
         <v>0</v>
       </c>
-      <c r="K34" s="24" t="n">
+      <c r="K34" s="25" t="n">
         <f aca="false">IF(I34="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I34)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>0</v>
       </c>
-      <c r="L34" s="24" t="n">
+      <c r="L34" s="25" t="n">
         <f aca="false">IF(I34="",-1,J34+(34-26)/1000000)</f>
         <v>-1</v>
       </c>
+      <c r="M34" s="26" t="n">
+        <f aca="false">IF(B34&lt;&gt;"",F34,M33)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="21" t="n">
+      <c r="A35" s="22" t="n">
         <v>27</v>
       </c>
       <c r="B35" s="10" t="str">
         <f aca="false">IF(INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A35),$L$9:$L$38,0))&lt;=0,"",INDEX($I$9:$I$38,MATCH(LARGE($L$9:$L$38,A35),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="C35" s="22" t="str">
+      <c r="C35" s="23" t="str">
         <f aca="false">IF(B35="","",INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A35),$L$9:$L$38,0)))</f>
         <v/>
       </c>
@@ -25477,40 +25619,44 @@
         <f aca="false">IF(B35="","",INDEX($K$9:$K$38,MATCH(LARGE($L$9:$L$38,A35),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="E35" s="23" t="str">
+      <c r="E35" s="24" t="str">
         <f aca="false">IF(OR(B35="",$B$6=0),"",C35/$B$6)</f>
         <v/>
       </c>
-      <c r="F35" s="23" t="str">
+      <c r="F35" s="24" t="str">
         <f aca="false">IF(OR(B35="",$B$6=0),"",SUM($C$9:C35)/$B$6)</f>
         <v/>
       </c>
-      <c r="I35" s="24" t="str">
+      <c r="I35" s="25" t="str">
         <f aca="false">IF(Setup!D31="","",IF(SUMPRODUCT(--(Setup!$D$4:D30=Setup!D31))&gt;0,"",Setup!D31))</f>
         <v/>
       </c>
-      <c r="J35" s="24" t="n">
+      <c r="J35" s="25" t="n">
         <f aca="false">IF(I35="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I35)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0),'Downtime Log'!$G$5:$G$1004))</f>
         <v>0</v>
       </c>
-      <c r="K35" s="24" t="n">
+      <c r="K35" s="25" t="n">
         <f aca="false">IF(I35="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I35)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>0</v>
       </c>
-      <c r="L35" s="24" t="n">
+      <c r="L35" s="25" t="n">
         <f aca="false">IF(I35="",-1,J35+(34-27)/1000000)</f>
         <v>-1</v>
       </c>
+      <c r="M35" s="26" t="n">
+        <f aca="false">IF(B35&lt;&gt;"",F35,M34)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="21" t="n">
+      <c r="A36" s="22" t="n">
         <v>28</v>
       </c>
       <c r="B36" s="10" t="str">
         <f aca="false">IF(INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A36),$L$9:$L$38,0))&lt;=0,"",INDEX($I$9:$I$38,MATCH(LARGE($L$9:$L$38,A36),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="C36" s="22" t="str">
+      <c r="C36" s="23" t="str">
         <f aca="false">IF(B36="","",INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A36),$L$9:$L$38,0)))</f>
         <v/>
       </c>
@@ -25518,40 +25664,44 @@
         <f aca="false">IF(B36="","",INDEX($K$9:$K$38,MATCH(LARGE($L$9:$L$38,A36),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="E36" s="23" t="str">
+      <c r="E36" s="24" t="str">
         <f aca="false">IF(OR(B36="",$B$6=0),"",C36/$B$6)</f>
         <v/>
       </c>
-      <c r="F36" s="23" t="str">
+      <c r="F36" s="24" t="str">
         <f aca="false">IF(OR(B36="",$B$6=0),"",SUM($C$9:C36)/$B$6)</f>
         <v/>
       </c>
-      <c r="I36" s="24" t="str">
+      <c r="I36" s="25" t="str">
         <f aca="false">IF(Setup!D32="","",IF(SUMPRODUCT(--(Setup!$D$4:D31=Setup!D32))&gt;0,"",Setup!D32))</f>
         <v/>
       </c>
-      <c r="J36" s="24" t="n">
+      <c r="J36" s="25" t="n">
         <f aca="false">IF(I36="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I36)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0),'Downtime Log'!$G$5:$G$1004))</f>
         <v>0</v>
       </c>
-      <c r="K36" s="24" t="n">
+      <c r="K36" s="25" t="n">
         <f aca="false">IF(I36="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I36)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>0</v>
       </c>
-      <c r="L36" s="24" t="n">
+      <c r="L36" s="25" t="n">
         <f aca="false">IF(I36="",-1,J36+(34-28)/1000000)</f>
         <v>-1</v>
       </c>
+      <c r="M36" s="26" t="n">
+        <f aca="false">IF(B36&lt;&gt;"",F36,M35)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="21" t="n">
+      <c r="A37" s="22" t="n">
         <v>29</v>
       </c>
       <c r="B37" s="10" t="str">
         <f aca="false">IF(INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A37),$L$9:$L$38,0))&lt;=0,"",INDEX($I$9:$I$38,MATCH(LARGE($L$9:$L$38,A37),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="C37" s="22" t="str">
+      <c r="C37" s="23" t="str">
         <f aca="false">IF(B37="","",INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A37),$L$9:$L$38,0)))</f>
         <v/>
       </c>
@@ -25559,40 +25709,44 @@
         <f aca="false">IF(B37="","",INDEX($K$9:$K$38,MATCH(LARGE($L$9:$L$38,A37),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="E37" s="23" t="str">
+      <c r="E37" s="24" t="str">
         <f aca="false">IF(OR(B37="",$B$6=0),"",C37/$B$6)</f>
         <v/>
       </c>
-      <c r="F37" s="23" t="str">
+      <c r="F37" s="24" t="str">
         <f aca="false">IF(OR(B37="",$B$6=0),"",SUM($C$9:C37)/$B$6)</f>
         <v/>
       </c>
-      <c r="I37" s="24" t="str">
+      <c r="I37" s="25" t="str">
         <f aca="false">IF(Setup!D33="","",IF(SUMPRODUCT(--(Setup!$D$4:D32=Setup!D33))&gt;0,"",Setup!D33))</f>
         <v/>
       </c>
-      <c r="J37" s="24" t="n">
+      <c r="J37" s="25" t="n">
         <f aca="false">IF(I37="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I37)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0),'Downtime Log'!$G$5:$G$1004))</f>
         <v>0</v>
       </c>
-      <c r="K37" s="24" t="n">
+      <c r="K37" s="25" t="n">
         <f aca="false">IF(I37="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I37)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>0</v>
       </c>
-      <c r="L37" s="24" t="n">
+      <c r="L37" s="25" t="n">
         <f aca="false">IF(I37="",-1,J37+(34-29)/1000000)</f>
         <v>-1</v>
       </c>
+      <c r="M37" s="26" t="n">
+        <f aca="false">IF(B37&lt;&gt;"",F37,M36)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="21" t="n">
+      <c r="A38" s="22" t="n">
         <v>30</v>
       </c>
       <c r="B38" s="10" t="str">
         <f aca="false">IF(INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A38),$L$9:$L$38,0))&lt;=0,"",INDEX($I$9:$I$38,MATCH(LARGE($L$9:$L$38,A38),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="C38" s="22" t="str">
+      <c r="C38" s="23" t="str">
         <f aca="false">IF(B38="","",INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A38),$L$9:$L$38,0)))</f>
         <v/>
       </c>
@@ -25600,29 +25754,33 @@
         <f aca="false">IF(B38="","",INDEX($K$9:$K$38,MATCH(LARGE($L$9:$L$38,A38),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="E38" s="23" t="str">
+      <c r="E38" s="24" t="str">
         <f aca="false">IF(OR(B38="",$B$6=0),"",C38/$B$6)</f>
         <v/>
       </c>
-      <c r="F38" s="23" t="str">
+      <c r="F38" s="24" t="str">
         <f aca="false">IF(OR(B38="",$B$6=0),"",SUM($C$9:C38)/$B$6)</f>
         <v/>
       </c>
-      <c r="I38" s="24" t="str">
+      <c r="I38" s="25" t="str">
         <f aca="false">IF(Setup!D34="","",IF(SUMPRODUCT(--(Setup!$D$4:D33=Setup!D34))&gt;0,"",Setup!D34))</f>
         <v/>
       </c>
-      <c r="J38" s="24" t="n">
+      <c r="J38" s="25" t="n">
         <f aca="false">IF(I38="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I38)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0),'Downtime Log'!$G$5:$G$1004))</f>
         <v>0</v>
       </c>
-      <c r="K38" s="24" t="n">
+      <c r="K38" s="25" t="n">
         <f aca="false">IF(I38="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I38)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>0</v>
       </c>
-      <c r="L38" s="24" t="n">
+      <c r="L38" s="25" t="n">
         <f aca="false">IF(I38="",-1,J38+(34-30)/1000000)</f>
         <v>-1</v>
+      </c>
+      <c r="M38" s="26" t="n">
+        <f aca="false">IF(B38&lt;&gt;"",F38,M37)</f>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -25690,7 +25848,7 @@
         <f aca="false">IF(Setup!A5="","",IF(SUMPRODUCT(--(Setup!$A$4:A4=Setup!A5))&gt;0,"",Setup!A5))</f>
         <v>Press 01</v>
       </c>
-      <c r="B5" s="22" t="n">
+      <c r="B5" s="23" t="n">
         <f aca="false">IF($A5="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A5)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004))</f>
         <v>105</v>
       </c>
@@ -25698,11 +25856,11 @@
         <f aca="false">IF($A5="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A5)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>3</v>
       </c>
-      <c r="D5" s="25" t="n">
+      <c r="D5" s="27" t="n">
         <f aca="false">IF(OR($A5="",N(C5)=0),"",B5/C5)</f>
         <v>35</v>
       </c>
-      <c r="E5" s="23" t="n">
+      <c r="E5" s="24" t="n">
         <f aca="false">IF(OR($A5="",$B$36=0),"",B5/$B$36)</f>
         <v>0.411764705882353</v>
       </c>
@@ -25712,7 +25870,7 @@
         <f aca="false">IF(Setup!A6="","",IF(SUMPRODUCT(--(Setup!$A$4:A5=Setup!A6))&gt;0,"",Setup!A6))</f>
         <v>CNC Lathe 02</v>
       </c>
-      <c r="B6" s="22" t="n">
+      <c r="B6" s="23" t="n">
         <f aca="false">IF($A6="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A6)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004))</f>
         <v>75</v>
       </c>
@@ -25720,11 +25878,11 @@
         <f aca="false">IF($A6="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A6)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>2</v>
       </c>
-      <c r="D6" s="25" t="n">
+      <c r="D6" s="27" t="n">
         <f aca="false">IF(OR($A6="",N(C6)=0),"",B6/C6)</f>
         <v>37.5</v>
       </c>
-      <c r="E6" s="23" t="n">
+      <c r="E6" s="24" t="n">
         <f aca="false">IF(OR($A6="",$B$36=0),"",B6/$B$36)</f>
         <v>0.294117647058824</v>
       </c>
@@ -25734,7 +25892,7 @@
         <f aca="false">IF(Setup!A7="","",IF(SUMPRODUCT(--(Setup!$A$4:A6=Setup!A7))&gt;0,"",Setup!A7))</f>
         <v>Packaging Line A</v>
       </c>
-      <c r="B7" s="22" t="n">
+      <c r="B7" s="23" t="n">
         <f aca="false">IF($A7="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A7)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004))</f>
         <v>75</v>
       </c>
@@ -25742,11 +25900,11 @@
         <f aca="false">IF($A7="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A7)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>2</v>
       </c>
-      <c r="D7" s="25" t="n">
+      <c r="D7" s="27" t="n">
         <f aca="false">IF(OR($A7="",N(C7)=0),"",B7/C7)</f>
         <v>37.5</v>
       </c>
-      <c r="E7" s="23" t="n">
+      <c r="E7" s="24" t="n">
         <f aca="false">IF(OR($A7="",$B$36=0),"",B7/$B$36)</f>
         <v>0.294117647058824</v>
       </c>
@@ -25756,7 +25914,7 @@
         <f aca="false">IF(Setup!A8="","",IF(SUMPRODUCT(--(Setup!$A$4:A7=Setup!A8))&gt;0,"",Setup!A8))</f>
         <v/>
       </c>
-      <c r="B8" s="22" t="str">
+      <c r="B8" s="23" t="str">
         <f aca="false">IF($A8="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A8)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004))</f>
         <v/>
       </c>
@@ -25764,11 +25922,11 @@
         <f aca="false">IF($A8="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A8)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v/>
       </c>
-      <c r="D8" s="25" t="str">
+      <c r="D8" s="27" t="str">
         <f aca="false">IF(OR($A8="",N(C8)=0),"",B8/C8)</f>
         <v/>
       </c>
-      <c r="E8" s="23" t="str">
+      <c r="E8" s="24" t="str">
         <f aca="false">IF(OR($A8="",$B$36=0),"",B8/$B$36)</f>
         <v/>
       </c>
@@ -25778,7 +25936,7 @@
         <f aca="false">IF(Setup!A9="","",IF(SUMPRODUCT(--(Setup!$A$4:A8=Setup!A9))&gt;0,"",Setup!A9))</f>
         <v/>
       </c>
-      <c r="B9" s="22" t="str">
+      <c r="B9" s="23" t="str">
         <f aca="false">IF($A9="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A9)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004))</f>
         <v/>
       </c>
@@ -25786,11 +25944,11 @@
         <f aca="false">IF($A9="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A9)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v/>
       </c>
-      <c r="D9" s="25" t="str">
+      <c r="D9" s="27" t="str">
         <f aca="false">IF(OR($A9="",N(C9)=0),"",B9/C9)</f>
         <v/>
       </c>
-      <c r="E9" s="23" t="str">
+      <c r="E9" s="24" t="str">
         <f aca="false">IF(OR($A9="",$B$36=0),"",B9/$B$36)</f>
         <v/>
       </c>
@@ -25800,7 +25958,7 @@
         <f aca="false">IF(Setup!A10="","",IF(SUMPRODUCT(--(Setup!$A$4:A9=Setup!A10))&gt;0,"",Setup!A10))</f>
         <v/>
       </c>
-      <c r="B10" s="22" t="str">
+      <c r="B10" s="23" t="str">
         <f aca="false">IF($A10="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A10)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004))</f>
         <v/>
       </c>
@@ -25808,11 +25966,11 @@
         <f aca="false">IF($A10="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A10)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v/>
       </c>
-      <c r="D10" s="25" t="str">
+      <c r="D10" s="27" t="str">
         <f aca="false">IF(OR($A10="",N(C10)=0),"",B10/C10)</f>
         <v/>
       </c>
-      <c r="E10" s="23" t="str">
+      <c r="E10" s="24" t="str">
         <f aca="false">IF(OR($A10="",$B$36=0),"",B10/$B$36)</f>
         <v/>
       </c>
@@ -25822,7 +25980,7 @@
         <f aca="false">IF(Setup!A11="","",IF(SUMPRODUCT(--(Setup!$A$4:A10=Setup!A11))&gt;0,"",Setup!A11))</f>
         <v/>
       </c>
-      <c r="B11" s="22" t="str">
+      <c r="B11" s="23" t="str">
         <f aca="false">IF($A11="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A11)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004))</f>
         <v/>
       </c>
@@ -25830,11 +25988,11 @@
         <f aca="false">IF($A11="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A11)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v/>
       </c>
-      <c r="D11" s="25" t="str">
+      <c r="D11" s="27" t="str">
         <f aca="false">IF(OR($A11="",N(C11)=0),"",B11/C11)</f>
         <v/>
       </c>
-      <c r="E11" s="23" t="str">
+      <c r="E11" s="24" t="str">
         <f aca="false">IF(OR($A11="",$B$36=0),"",B11/$B$36)</f>
         <v/>
       </c>
@@ -25844,7 +26002,7 @@
         <f aca="false">IF(Setup!A12="","",IF(SUMPRODUCT(--(Setup!$A$4:A11=Setup!A12))&gt;0,"",Setup!A12))</f>
         <v/>
       </c>
-      <c r="B12" s="22" t="str">
+      <c r="B12" s="23" t="str">
         <f aca="false">IF($A12="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A12)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004))</f>
         <v/>
       </c>
@@ -25852,11 +26010,11 @@
         <f aca="false">IF($A12="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A12)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v/>
       </c>
-      <c r="D12" s="25" t="str">
+      <c r="D12" s="27" t="str">
         <f aca="false">IF(OR($A12="",N(C12)=0),"",B12/C12)</f>
         <v/>
       </c>
-      <c r="E12" s="23" t="str">
+      <c r="E12" s="24" t="str">
         <f aca="false">IF(OR($A12="",$B$36=0),"",B12/$B$36)</f>
         <v/>
       </c>
@@ -25866,7 +26024,7 @@
         <f aca="false">IF(Setup!A13="","",IF(SUMPRODUCT(--(Setup!$A$4:A12=Setup!A13))&gt;0,"",Setup!A13))</f>
         <v/>
       </c>
-      <c r="B13" s="22" t="str">
+      <c r="B13" s="23" t="str">
         <f aca="false">IF($A13="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A13)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004))</f>
         <v/>
       </c>
@@ -25874,11 +26032,11 @@
         <f aca="false">IF($A13="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A13)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v/>
       </c>
-      <c r="D13" s="25" t="str">
+      <c r="D13" s="27" t="str">
         <f aca="false">IF(OR($A13="",N(C13)=0),"",B13/C13)</f>
         <v/>
       </c>
-      <c r="E13" s="23" t="str">
+      <c r="E13" s="24" t="str">
         <f aca="false">IF(OR($A13="",$B$36=0),"",B13/$B$36)</f>
         <v/>
       </c>
@@ -25888,7 +26046,7 @@
         <f aca="false">IF(Setup!A14="","",IF(SUMPRODUCT(--(Setup!$A$4:A13=Setup!A14))&gt;0,"",Setup!A14))</f>
         <v/>
       </c>
-      <c r="B14" s="22" t="str">
+      <c r="B14" s="23" t="str">
         <f aca="false">IF($A14="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A14)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004))</f>
         <v/>
       </c>
@@ -25896,11 +26054,11 @@
         <f aca="false">IF($A14="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A14)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v/>
       </c>
-      <c r="D14" s="25" t="str">
+      <c r="D14" s="27" t="str">
         <f aca="false">IF(OR($A14="",N(C14)=0),"",B14/C14)</f>
         <v/>
       </c>
-      <c r="E14" s="23" t="str">
+      <c r="E14" s="24" t="str">
         <f aca="false">IF(OR($A14="",$B$36=0),"",B14/$B$36)</f>
         <v/>
       </c>
@@ -25910,7 +26068,7 @@
         <f aca="false">IF(Setup!A15="","",IF(SUMPRODUCT(--(Setup!$A$4:A14=Setup!A15))&gt;0,"",Setup!A15))</f>
         <v/>
       </c>
-      <c r="B15" s="22" t="str">
+      <c r="B15" s="23" t="str">
         <f aca="false">IF($A15="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A15)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004))</f>
         <v/>
       </c>
@@ -25918,11 +26076,11 @@
         <f aca="false">IF($A15="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A15)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v/>
       </c>
-      <c r="D15" s="25" t="str">
+      <c r="D15" s="27" t="str">
         <f aca="false">IF(OR($A15="",N(C15)=0),"",B15/C15)</f>
         <v/>
       </c>
-      <c r="E15" s="23" t="str">
+      <c r="E15" s="24" t="str">
         <f aca="false">IF(OR($A15="",$B$36=0),"",B15/$B$36)</f>
         <v/>
       </c>
@@ -25932,7 +26090,7 @@
         <f aca="false">IF(Setup!A16="","",IF(SUMPRODUCT(--(Setup!$A$4:A15=Setup!A16))&gt;0,"",Setup!A16))</f>
         <v/>
       </c>
-      <c r="B16" s="22" t="str">
+      <c r="B16" s="23" t="str">
         <f aca="false">IF($A16="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A16)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004))</f>
         <v/>
       </c>
@@ -25940,11 +26098,11 @@
         <f aca="false">IF($A16="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A16)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v/>
       </c>
-      <c r="D16" s="25" t="str">
+      <c r="D16" s="27" t="str">
         <f aca="false">IF(OR($A16="",N(C16)=0),"",B16/C16)</f>
         <v/>
       </c>
-      <c r="E16" s="23" t="str">
+      <c r="E16" s="24" t="str">
         <f aca="false">IF(OR($A16="",$B$36=0),"",B16/$B$36)</f>
         <v/>
       </c>
@@ -25954,7 +26112,7 @@
         <f aca="false">IF(Setup!A17="","",IF(SUMPRODUCT(--(Setup!$A$4:A16=Setup!A17))&gt;0,"",Setup!A17))</f>
         <v/>
       </c>
-      <c r="B17" s="22" t="str">
+      <c r="B17" s="23" t="str">
         <f aca="false">IF($A17="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A17)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004))</f>
         <v/>
       </c>
@@ -25962,11 +26120,11 @@
         <f aca="false">IF($A17="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A17)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v/>
       </c>
-      <c r="D17" s="25" t="str">
+      <c r="D17" s="27" t="str">
         <f aca="false">IF(OR($A17="",N(C17)=0),"",B17/C17)</f>
         <v/>
       </c>
-      <c r="E17" s="23" t="str">
+      <c r="E17" s="24" t="str">
         <f aca="false">IF(OR($A17="",$B$36=0),"",B17/$B$36)</f>
         <v/>
       </c>
@@ -25976,7 +26134,7 @@
         <f aca="false">IF(Setup!A18="","",IF(SUMPRODUCT(--(Setup!$A$4:A17=Setup!A18))&gt;0,"",Setup!A18))</f>
         <v/>
       </c>
-      <c r="B18" s="22" t="str">
+      <c r="B18" s="23" t="str">
         <f aca="false">IF($A18="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A18)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004))</f>
         <v/>
       </c>
@@ -25984,11 +26142,11 @@
         <f aca="false">IF($A18="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A18)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v/>
       </c>
-      <c r="D18" s="25" t="str">
+      <c r="D18" s="27" t="str">
         <f aca="false">IF(OR($A18="",N(C18)=0),"",B18/C18)</f>
         <v/>
       </c>
-      <c r="E18" s="23" t="str">
+      <c r="E18" s="24" t="str">
         <f aca="false">IF(OR($A18="",$B$36=0),"",B18/$B$36)</f>
         <v/>
       </c>
@@ -25998,7 +26156,7 @@
         <f aca="false">IF(Setup!A19="","",IF(SUMPRODUCT(--(Setup!$A$4:A18=Setup!A19))&gt;0,"",Setup!A19))</f>
         <v/>
       </c>
-      <c r="B19" s="22" t="str">
+      <c r="B19" s="23" t="str">
         <f aca="false">IF($A19="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A19)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004))</f>
         <v/>
       </c>
@@ -26006,11 +26164,11 @@
         <f aca="false">IF($A19="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A19)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v/>
       </c>
-      <c r="D19" s="25" t="str">
+      <c r="D19" s="27" t="str">
         <f aca="false">IF(OR($A19="",N(C19)=0),"",B19/C19)</f>
         <v/>
       </c>
-      <c r="E19" s="23" t="str">
+      <c r="E19" s="24" t="str">
         <f aca="false">IF(OR($A19="",$B$36=0),"",B19/$B$36)</f>
         <v/>
       </c>
@@ -26020,7 +26178,7 @@
         <f aca="false">IF(Setup!A20="","",IF(SUMPRODUCT(--(Setup!$A$4:A19=Setup!A20))&gt;0,"",Setup!A20))</f>
         <v/>
       </c>
-      <c r="B20" s="22" t="str">
+      <c r="B20" s="23" t="str">
         <f aca="false">IF($A20="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A20)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004))</f>
         <v/>
       </c>
@@ -26028,11 +26186,11 @@
         <f aca="false">IF($A20="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A20)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v/>
       </c>
-      <c r="D20" s="25" t="str">
+      <c r="D20" s="27" t="str">
         <f aca="false">IF(OR($A20="",N(C20)=0),"",B20/C20)</f>
         <v/>
       </c>
-      <c r="E20" s="23" t="str">
+      <c r="E20" s="24" t="str">
         <f aca="false">IF(OR($A20="",$B$36=0),"",B20/$B$36)</f>
         <v/>
       </c>
@@ -26042,7 +26200,7 @@
         <f aca="false">IF(Setup!A21="","",IF(SUMPRODUCT(--(Setup!$A$4:A20=Setup!A21))&gt;0,"",Setup!A21))</f>
         <v/>
       </c>
-      <c r="B21" s="22" t="str">
+      <c r="B21" s="23" t="str">
         <f aca="false">IF($A21="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A21)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004))</f>
         <v/>
       </c>
@@ -26050,11 +26208,11 @@
         <f aca="false">IF($A21="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A21)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v/>
       </c>
-      <c r="D21" s="25" t="str">
+      <c r="D21" s="27" t="str">
         <f aca="false">IF(OR($A21="",N(C21)=0),"",B21/C21)</f>
         <v/>
       </c>
-      <c r="E21" s="23" t="str">
+      <c r="E21" s="24" t="str">
         <f aca="false">IF(OR($A21="",$B$36=0),"",B21/$B$36)</f>
         <v/>
       </c>
@@ -26064,7 +26222,7 @@
         <f aca="false">IF(Setup!A22="","",IF(SUMPRODUCT(--(Setup!$A$4:A21=Setup!A22))&gt;0,"",Setup!A22))</f>
         <v/>
       </c>
-      <c r="B22" s="22" t="str">
+      <c r="B22" s="23" t="str">
         <f aca="false">IF($A22="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A22)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004))</f>
         <v/>
       </c>
@@ -26072,11 +26230,11 @@
         <f aca="false">IF($A22="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A22)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v/>
       </c>
-      <c r="D22" s="25" t="str">
+      <c r="D22" s="27" t="str">
         <f aca="false">IF(OR($A22="",N(C22)=0),"",B22/C22)</f>
         <v/>
       </c>
-      <c r="E22" s="23" t="str">
+      <c r="E22" s="24" t="str">
         <f aca="false">IF(OR($A22="",$B$36=0),"",B22/$B$36)</f>
         <v/>
       </c>
@@ -26086,7 +26244,7 @@
         <f aca="false">IF(Setup!A23="","",IF(SUMPRODUCT(--(Setup!$A$4:A22=Setup!A23))&gt;0,"",Setup!A23))</f>
         <v/>
       </c>
-      <c r="B23" s="22" t="str">
+      <c r="B23" s="23" t="str">
         <f aca="false">IF($A23="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A23)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004))</f>
         <v/>
       </c>
@@ -26094,11 +26252,11 @@
         <f aca="false">IF($A23="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A23)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v/>
       </c>
-      <c r="D23" s="25" t="str">
+      <c r="D23" s="27" t="str">
         <f aca="false">IF(OR($A23="",N(C23)=0),"",B23/C23)</f>
         <v/>
       </c>
-      <c r="E23" s="23" t="str">
+      <c r="E23" s="24" t="str">
         <f aca="false">IF(OR($A23="",$B$36=0),"",B23/$B$36)</f>
         <v/>
       </c>
@@ -26108,7 +26266,7 @@
         <f aca="false">IF(Setup!A24="","",IF(SUMPRODUCT(--(Setup!$A$4:A23=Setup!A24))&gt;0,"",Setup!A24))</f>
         <v/>
       </c>
-      <c r="B24" s="22" t="str">
+      <c r="B24" s="23" t="str">
         <f aca="false">IF($A24="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A24)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004))</f>
         <v/>
       </c>
@@ -26116,11 +26274,11 @@
         <f aca="false">IF($A24="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A24)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v/>
       </c>
-      <c r="D24" s="25" t="str">
+      <c r="D24" s="27" t="str">
         <f aca="false">IF(OR($A24="",N(C24)=0),"",B24/C24)</f>
         <v/>
       </c>
-      <c r="E24" s="23" t="str">
+      <c r="E24" s="24" t="str">
         <f aca="false">IF(OR($A24="",$B$36=0),"",B24/$B$36)</f>
         <v/>
       </c>
@@ -26130,7 +26288,7 @@
         <f aca="false">IF(Setup!A25="","",IF(SUMPRODUCT(--(Setup!$A$4:A24=Setup!A25))&gt;0,"",Setup!A25))</f>
         <v/>
       </c>
-      <c r="B25" s="22" t="str">
+      <c r="B25" s="23" t="str">
         <f aca="false">IF($A25="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A25)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004))</f>
         <v/>
       </c>
@@ -26138,11 +26296,11 @@
         <f aca="false">IF($A25="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A25)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v/>
       </c>
-      <c r="D25" s="25" t="str">
+      <c r="D25" s="27" t="str">
         <f aca="false">IF(OR($A25="",N(C25)=0),"",B25/C25)</f>
         <v/>
       </c>
-      <c r="E25" s="23" t="str">
+      <c r="E25" s="24" t="str">
         <f aca="false">IF(OR($A25="",$B$36=0),"",B25/$B$36)</f>
         <v/>
       </c>
@@ -26152,7 +26310,7 @@
         <f aca="false">IF(Setup!A26="","",IF(SUMPRODUCT(--(Setup!$A$4:A25=Setup!A26))&gt;0,"",Setup!A26))</f>
         <v/>
       </c>
-      <c r="B26" s="22" t="str">
+      <c r="B26" s="23" t="str">
         <f aca="false">IF($A26="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A26)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004))</f>
         <v/>
       </c>
@@ -26160,11 +26318,11 @@
         <f aca="false">IF($A26="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A26)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v/>
       </c>
-      <c r="D26" s="25" t="str">
+      <c r="D26" s="27" t="str">
         <f aca="false">IF(OR($A26="",N(C26)=0),"",B26/C26)</f>
         <v/>
       </c>
-      <c r="E26" s="23" t="str">
+      <c r="E26" s="24" t="str">
         <f aca="false">IF(OR($A26="",$B$36=0),"",B26/$B$36)</f>
         <v/>
       </c>
@@ -26174,7 +26332,7 @@
         <f aca="false">IF(Setup!A27="","",IF(SUMPRODUCT(--(Setup!$A$4:A26=Setup!A27))&gt;0,"",Setup!A27))</f>
         <v/>
       </c>
-      <c r="B27" s="22" t="str">
+      <c r="B27" s="23" t="str">
         <f aca="false">IF($A27="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A27)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004))</f>
         <v/>
       </c>
@@ -26182,11 +26340,11 @@
         <f aca="false">IF($A27="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A27)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v/>
       </c>
-      <c r="D27" s="25" t="str">
+      <c r="D27" s="27" t="str">
         <f aca="false">IF(OR($A27="",N(C27)=0),"",B27/C27)</f>
         <v/>
       </c>
-      <c r="E27" s="23" t="str">
+      <c r="E27" s="24" t="str">
         <f aca="false">IF(OR($A27="",$B$36=0),"",B27/$B$36)</f>
         <v/>
       </c>
@@ -26196,7 +26354,7 @@
         <f aca="false">IF(Setup!A28="","",IF(SUMPRODUCT(--(Setup!$A$4:A27=Setup!A28))&gt;0,"",Setup!A28))</f>
         <v/>
       </c>
-      <c r="B28" s="22" t="str">
+      <c r="B28" s="23" t="str">
         <f aca="false">IF($A28="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A28)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004))</f>
         <v/>
       </c>
@@ -26204,11 +26362,11 @@
         <f aca="false">IF($A28="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A28)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v/>
       </c>
-      <c r="D28" s="25" t="str">
+      <c r="D28" s="27" t="str">
         <f aca="false">IF(OR($A28="",N(C28)=0),"",B28/C28)</f>
         <v/>
       </c>
-      <c r="E28" s="23" t="str">
+      <c r="E28" s="24" t="str">
         <f aca="false">IF(OR($A28="",$B$36=0),"",B28/$B$36)</f>
         <v/>
       </c>
@@ -26218,7 +26376,7 @@
         <f aca="false">IF(Setup!A29="","",IF(SUMPRODUCT(--(Setup!$A$4:A28=Setup!A29))&gt;0,"",Setup!A29))</f>
         <v/>
       </c>
-      <c r="B29" s="22" t="str">
+      <c r="B29" s="23" t="str">
         <f aca="false">IF($A29="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A29)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004))</f>
         <v/>
       </c>
@@ -26226,11 +26384,11 @@
         <f aca="false">IF($A29="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A29)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v/>
       </c>
-      <c r="D29" s="25" t="str">
+      <c r="D29" s="27" t="str">
         <f aca="false">IF(OR($A29="",N(C29)=0),"",B29/C29)</f>
         <v/>
       </c>
-      <c r="E29" s="23" t="str">
+      <c r="E29" s="24" t="str">
         <f aca="false">IF(OR($A29="",$B$36=0),"",B29/$B$36)</f>
         <v/>
       </c>
@@ -26240,7 +26398,7 @@
         <f aca="false">IF(Setup!A30="","",IF(SUMPRODUCT(--(Setup!$A$4:A29=Setup!A30))&gt;0,"",Setup!A30))</f>
         <v/>
       </c>
-      <c r="B30" s="22" t="str">
+      <c r="B30" s="23" t="str">
         <f aca="false">IF($A30="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A30)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004))</f>
         <v/>
       </c>
@@ -26248,11 +26406,11 @@
         <f aca="false">IF($A30="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A30)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v/>
       </c>
-      <c r="D30" s="25" t="str">
+      <c r="D30" s="27" t="str">
         <f aca="false">IF(OR($A30="",N(C30)=0),"",B30/C30)</f>
         <v/>
       </c>
-      <c r="E30" s="23" t="str">
+      <c r="E30" s="24" t="str">
         <f aca="false">IF(OR($A30="",$B$36=0),"",B30/$B$36)</f>
         <v/>
       </c>
@@ -26262,7 +26420,7 @@
         <f aca="false">IF(Setup!A31="","",IF(SUMPRODUCT(--(Setup!$A$4:A30=Setup!A31))&gt;0,"",Setup!A31))</f>
         <v/>
       </c>
-      <c r="B31" s="22" t="str">
+      <c r="B31" s="23" t="str">
         <f aca="false">IF($A31="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A31)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004))</f>
         <v/>
       </c>
@@ -26270,11 +26428,11 @@
         <f aca="false">IF($A31="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A31)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v/>
       </c>
-      <c r="D31" s="25" t="str">
+      <c r="D31" s="27" t="str">
         <f aca="false">IF(OR($A31="",N(C31)=0),"",B31/C31)</f>
         <v/>
       </c>
-      <c r="E31" s="23" t="str">
+      <c r="E31" s="24" t="str">
         <f aca="false">IF(OR($A31="",$B$36=0),"",B31/$B$36)</f>
         <v/>
       </c>
@@ -26284,7 +26442,7 @@
         <f aca="false">IF(Setup!A32="","",IF(SUMPRODUCT(--(Setup!$A$4:A31=Setup!A32))&gt;0,"",Setup!A32))</f>
         <v/>
       </c>
-      <c r="B32" s="22" t="str">
+      <c r="B32" s="23" t="str">
         <f aca="false">IF($A32="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A32)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004))</f>
         <v/>
       </c>
@@ -26292,11 +26450,11 @@
         <f aca="false">IF($A32="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A32)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v/>
       </c>
-      <c r="D32" s="25" t="str">
+      <c r="D32" s="27" t="str">
         <f aca="false">IF(OR($A32="",N(C32)=0),"",B32/C32)</f>
         <v/>
       </c>
-      <c r="E32" s="23" t="str">
+      <c r="E32" s="24" t="str">
         <f aca="false">IF(OR($A32="",$B$36=0),"",B32/$B$36)</f>
         <v/>
       </c>
@@ -26306,7 +26464,7 @@
         <f aca="false">IF(Setup!A33="","",IF(SUMPRODUCT(--(Setup!$A$4:A32=Setup!A33))&gt;0,"",Setup!A33))</f>
         <v/>
       </c>
-      <c r="B33" s="22" t="str">
+      <c r="B33" s="23" t="str">
         <f aca="false">IF($A33="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A33)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004))</f>
         <v/>
       </c>
@@ -26314,11 +26472,11 @@
         <f aca="false">IF($A33="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A33)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v/>
       </c>
-      <c r="D33" s="25" t="str">
+      <c r="D33" s="27" t="str">
         <f aca="false">IF(OR($A33="",N(C33)=0),"",B33/C33)</f>
         <v/>
       </c>
-      <c r="E33" s="23" t="str">
+      <c r="E33" s="24" t="str">
         <f aca="false">IF(OR($A33="",$B$36=0),"",B33/$B$36)</f>
         <v/>
       </c>
@@ -26328,7 +26486,7 @@
         <f aca="false">IF(Setup!A34="","",IF(SUMPRODUCT(--(Setup!$A$4:A33=Setup!A34))&gt;0,"",Setup!A34))</f>
         <v/>
       </c>
-      <c r="B34" s="22" t="str">
+      <c r="B34" s="23" t="str">
         <f aca="false">IF($A34="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A34)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004))</f>
         <v/>
       </c>
@@ -26336,11 +26494,11 @@
         <f aca="false">IF($A34="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A34)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v/>
       </c>
-      <c r="D34" s="25" t="str">
+      <c r="D34" s="27" t="str">
         <f aca="false">IF(OR($A34="",N(C34)=0),"",B34/C34)</f>
         <v/>
       </c>
-      <c r="E34" s="23" t="str">
+      <c r="E34" s="24" t="str">
         <f aca="false">IF(OR($A34="",$B$36=0),"",B34/$B$36)</f>
         <v/>
       </c>
@@ -26349,7 +26507,7 @@
       <c r="A35" s="10" t="s">
         <v>84</v>
       </c>
-      <c r="B35" s="22" t="n">
+      <c r="B35" s="23" t="n">
         <f aca="false">B36-SUM(B5:B34)</f>
         <v>0</v>
       </c>
@@ -26357,32 +26515,32 @@
         <f aca="false">SUMPRODUCT(('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0))-SUM(C5:C34)</f>
         <v>0</v>
       </c>
-      <c r="D35" s="25" t="str">
+      <c r="D35" s="27" t="str">
         <f aca="false">IF(OR($A35="",N(C35)=0),"",B35/C35)</f>
         <v/>
       </c>
-      <c r="E35" s="23" t="n">
+      <c r="E35" s="24" t="n">
         <f aca="false">IF(OR($A35="",$B$36=0),"",B35/$B$36)</f>
         <v>0</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="26" t="s">
+      <c r="A36" s="28" t="s">
         <v>85</v>
       </c>
-      <c r="B36" s="27" t="n">
+      <c r="B36" s="29" t="n">
         <f aca="false">SUMPRODUCT(('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004)</f>
         <v>255</v>
       </c>
-      <c r="C36" s="28" t="n">
+      <c r="C36" s="30" t="n">
         <f aca="false">SUMPRODUCT(('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0))</f>
         <v>7</v>
       </c>
-      <c r="D36" s="29" t="n">
+      <c r="D36" s="31" t="n">
         <f aca="false">IF(OR($A36="",N(C36)=0),"",B36/C36)</f>
         <v>36.4285714285714</v>
       </c>
-      <c r="E36" s="30" t="n">
+      <c r="E36" s="32" t="n">
         <f aca="false">IF(OR($A36="",$B$36=0),"",B36/$B$36)</f>
         <v>1</v>
       </c>

</xml_diff>

<commit_message>
Excel for the web passes; Pareto chart fix for Excel (#50)
* Hold: Pareto chart fix for Excel, plus Excel for the web results (not for merge yet)

- Pareto line plots a helper column that carries the last cumulative % forward,
  so empty rows no longer plot as 0 in Excel. Found uncommitted in the workspace;
  passes LibreOffice 188/188, not yet checked in Excel.
- Excel for the web: 188/188 suite checks pass (results-excel-web.json).

On hold pending the owner's decision in #48 (tripwire). No PR opened.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FtnizgcUQQWB874QqXt4YR

* Excel for the web passes; Pareto chart fix verified in Excel; refresh previews and guides

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FtnizgcUQQWB874QqXt4YR

---------

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/products/manufacturing-templates/dist/Downtime-Log-and-Pareto.xlsx
+++ b/products/manufacturing-templates/dist/Downtime-Log-and-Pareto.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="86">
   <si>
     <t xml:space="preserve">Downtime Log &amp; Pareto</t>
   </si>
@@ -302,7 +302,7 @@
     <numFmt numFmtId="170" formatCode="0%"/>
     <numFmt numFmtId="171" formatCode="0.0"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="18">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -410,6 +410,12 @@
       <family val="2"/>
     </font>
     <font>
+      <sz val="8"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
@@ -498,7 +504,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="33">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -583,6 +589,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -596,6 +606,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -859,8 +873,8 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="7198020"/>
-        <c:axId val="6383468"/>
+        <c:axId val="30367123"/>
+        <c:axId val="10482130"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -870,7 +884,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>Pareto!F8</c:f>
+              <c:f>Pareto!M8</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -964,7 +978,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Pareto!$F$9:$F$20</c:f>
+              <c:f>Pareto!$M$9:$M$20</c:f>
               <c:numCache>
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="12"/>
@@ -983,6 +997,27 @@
                 <c:pt idx="4">
                   <c:v>1</c:v>
                 </c:pt>
+                <c:pt idx="5">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>1</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -996,11 +1031,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="62506310"/>
-        <c:axId val="68067979"/>
+        <c:axId val="42842550"/>
+        <c:axId val="48986869"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="7198020"/>
+        <c:axId val="30367123"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1019,11 +1054,11 @@
           </a:ln>
         </c:spPr>
         <c:txPr>
-          <a:bodyPr/>
+          <a:bodyPr rot="-2700000"/>
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+              <a:defRPr b="0" sz="800" spc="-1" strike="noStrike">
                 <a:solidFill>
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
@@ -1032,7 +1067,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="6383468"/>
+        <c:crossAx val="10482130"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1040,7 +1075,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="6383468"/>
+        <c:axId val="10482130"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1116,16 +1151,16 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="7198020"/>
+        <c:crossAx val="30367123"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:catAx>
-        <c:axId val="62506310"/>
+        <c:axId val="42842550"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
-        <c:delete val="0"/>
+        <c:delete val="1"/>
         <c:axPos val="t"/>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
@@ -1153,15 +1188,14 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="68067979"/>
-        <c:crosses val="autoZero"/>
+        <c:crossAx val="48986869"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="68067979"/>
+        <c:axId val="48986869"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -1229,7 +1263,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="62506310"/>
+        <c:crossAx val="42842550"/>
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1264,7 +1298,7 @@
         </a:p>
       </c:txPr>
     </c:legend>
-    <c:plotVisOnly val="1"/>
+    <c:plotVisOnly val="0"/>
     <c:dispBlanksAs val="gap"/>
   </c:chart>
   <c:spPr>
@@ -1285,16 +1319,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>7</xdr:col>
+      <xdr:col>13</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>130680</xdr:rowOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>340200</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>23</xdr:col>
-      <xdr:colOff>261720</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>112680</xdr:rowOff>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>473400</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>131760</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1302,7 +1336,7 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="7518960" y="380880"/>
+        <a:off x="7730640" y="1733400"/>
         <a:ext cx="7199640" cy="3239640"/>
       </xdr:xfrm>
       <a:graphic>
@@ -24290,7 +24324,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L38"/>
+  <dimension ref="A1:M38"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
@@ -24304,6 +24338,7 @@
     <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="10" min="10" style="0" width="11"/>
     <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="11" min="11" style="0" width="9"/>
     <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="12" min="12" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="13" min="13" style="0" width="13"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -24394,16 +24429,19 @@
       <c r="L8" s="20" t="s">
         <v>78</v>
       </c>
+      <c r="M8" s="21" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="21" t="n">
+      <c r="A9" s="22" t="n">
         <v>1</v>
       </c>
       <c r="B9" s="10" t="str">
         <f aca="false">IF(INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A9),$L$9:$L$38,0))&lt;=0,"",INDEX($I$9:$I$38,MATCH(LARGE($L$9:$L$38,A9),$L$9:$L$38,0)))</f>
         <v>Mechanical breakdown</v>
       </c>
-      <c r="C9" s="22" t="n">
+      <c r="C9" s="23" t="n">
         <f aca="false">IF(B9="","",INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A9),$L$9:$L$38,0)))</f>
         <v>100</v>
       </c>
@@ -24411,40 +24449,44 @@
         <f aca="false">IF(B9="","",INDEX($K$9:$K$38,MATCH(LARGE($L$9:$L$38,A9),$L$9:$L$38,0)))</f>
         <v>2</v>
       </c>
-      <c r="E9" s="23" t="n">
+      <c r="E9" s="24" t="n">
         <f aca="false">IF(OR(B9="",$B$6=0),"",C9/$B$6)</f>
         <v>0.392156862745098</v>
       </c>
-      <c r="F9" s="23" t="n">
+      <c r="F9" s="24" t="n">
         <f aca="false">IF(OR(B9="",$B$6=0),"",SUM($C$9:C9)/$B$6)</f>
         <v>0.392156862745098</v>
       </c>
-      <c r="I9" s="24" t="str">
+      <c r="I9" s="25" t="str">
         <f aca="false">IF(Setup!D5="","",IF(SUMPRODUCT(--(Setup!$D$4:D4=Setup!D5))&gt;0,"",Setup!D5))</f>
         <v>Mechanical breakdown</v>
       </c>
-      <c r="J9" s="24" t="n">
+      <c r="J9" s="25" t="n">
         <f aca="false">IF(I9="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I9)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0),'Downtime Log'!$G$5:$G$1004))</f>
         <v>100</v>
       </c>
-      <c r="K9" s="24" t="n">
+      <c r="K9" s="25" t="n">
         <f aca="false">IF(I9="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I9)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>2</v>
       </c>
-      <c r="L9" s="24" t="n">
+      <c r="L9" s="25" t="n">
         <f aca="false">IF(I9="",-1,J9+(34-1)/1000000)</f>
         <v>100.000033</v>
       </c>
+      <c r="M9" s="26" t="n">
+        <f aca="false">IF(B9&lt;&gt;"",F9,"")</f>
+        <v>0.392156862745098</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="21" t="n">
+      <c r="A10" s="22" t="n">
         <v>2</v>
       </c>
       <c r="B10" s="10" t="str">
         <f aca="false">IF(INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A10),$L$9:$L$38,0))&lt;=0,"",INDEX($I$9:$I$38,MATCH(LARGE($L$9:$L$38,A10),$L$9:$L$38,0)))</f>
         <v>Changeover / setup</v>
       </c>
-      <c r="C10" s="22" t="n">
+      <c r="C10" s="23" t="n">
         <f aca="false">IF(B10="","",INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A10),$L$9:$L$38,0)))</f>
         <v>65</v>
       </c>
@@ -24452,40 +24494,44 @@
         <f aca="false">IF(B10="","",INDEX($K$9:$K$38,MATCH(LARGE($L$9:$L$38,A10),$L$9:$L$38,0)))</f>
         <v>2</v>
       </c>
-      <c r="E10" s="23" t="n">
+      <c r="E10" s="24" t="n">
         <f aca="false">IF(OR(B10="",$B$6=0),"",C10/$B$6)</f>
         <v>0.254901960784314</v>
       </c>
-      <c r="F10" s="23" t="n">
+      <c r="F10" s="24" t="n">
         <f aca="false">IF(OR(B10="",$B$6=0),"",SUM($C$9:C10)/$B$6)</f>
         <v>0.647058823529412</v>
       </c>
-      <c r="I10" s="24" t="str">
+      <c r="I10" s="25" t="str">
         <f aca="false">IF(Setup!D6="","",IF(SUMPRODUCT(--(Setup!$D$4:D5=Setup!D6))&gt;0,"",Setup!D6))</f>
         <v>Electrical / controls fault</v>
       </c>
-      <c r="J10" s="24" t="n">
+      <c r="J10" s="25" t="n">
         <f aca="false">IF(I10="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I10)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0),'Downtime Log'!$G$5:$G$1004))</f>
         <v>0</v>
       </c>
-      <c r="K10" s="24" t="n">
+      <c r="K10" s="25" t="n">
         <f aca="false">IF(I10="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I10)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>0</v>
       </c>
-      <c r="L10" s="24" t="n">
+      <c r="L10" s="25" t="n">
         <f aca="false">IF(I10="",-1,J10+(34-2)/1000000)</f>
         <v>3.2E-005</v>
       </c>
+      <c r="M10" s="26" t="n">
+        <f aca="false">IF(B10&lt;&gt;"",F10,M9)</f>
+        <v>0.647058823529412</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="21" t="n">
+      <c r="A11" s="22" t="n">
         <v>3</v>
       </c>
       <c r="B11" s="10" t="str">
         <f aca="false">IF(INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A11),$L$9:$L$38,0))&lt;=0,"",INDEX($I$9:$I$38,MATCH(LARGE($L$9:$L$38,A11),$L$9:$L$38,0)))</f>
         <v>Tooling failure</v>
       </c>
-      <c r="C11" s="22" t="n">
+      <c r="C11" s="23" t="n">
         <f aca="false">IF(B11="","",INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A11),$L$9:$L$38,0)))</f>
         <v>60</v>
       </c>
@@ -24493,40 +24539,44 @@
         <f aca="false">IF(B11="","",INDEX($K$9:$K$38,MATCH(LARGE($L$9:$L$38,A11),$L$9:$L$38,0)))</f>
         <v>1</v>
       </c>
-      <c r="E11" s="23" t="n">
+      <c r="E11" s="24" t="n">
         <f aca="false">IF(OR(B11="",$B$6=0),"",C11/$B$6)</f>
         <v>0.235294117647059</v>
       </c>
-      <c r="F11" s="23" t="n">
+      <c r="F11" s="24" t="n">
         <f aca="false">IF(OR(B11="",$B$6=0),"",SUM($C$9:C11)/$B$6)</f>
         <v>0.882352941176471</v>
       </c>
-      <c r="I11" s="24" t="str">
+      <c r="I11" s="25" t="str">
         <f aca="false">IF(Setup!D7="","",IF(SUMPRODUCT(--(Setup!$D$4:D6=Setup!D7))&gt;0,"",Setup!D7))</f>
         <v>Tooling failure</v>
       </c>
-      <c r="J11" s="24" t="n">
+      <c r="J11" s="25" t="n">
         <f aca="false">IF(I11="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I11)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0),'Downtime Log'!$G$5:$G$1004))</f>
         <v>60</v>
       </c>
-      <c r="K11" s="24" t="n">
+      <c r="K11" s="25" t="n">
         <f aca="false">IF(I11="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I11)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>1</v>
       </c>
-      <c r="L11" s="24" t="n">
+      <c r="L11" s="25" t="n">
         <f aca="false">IF(I11="",-1,J11+(34-3)/1000000)</f>
         <v>60.000031</v>
       </c>
+      <c r="M11" s="26" t="n">
+        <f aca="false">IF(B11&lt;&gt;"",F11,M10)</f>
+        <v>0.882352941176471</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="21" t="n">
+      <c r="A12" s="22" t="n">
         <v>4</v>
       </c>
       <c r="B12" s="10" t="str">
         <f aca="false">IF(INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A12),$L$9:$L$38,0))&lt;=0,"",INDEX($I$9:$I$38,MATCH(LARGE($L$9:$L$38,A12),$L$9:$L$38,0)))</f>
         <v>Waiting for material</v>
       </c>
-      <c r="C12" s="22" t="n">
+      <c r="C12" s="23" t="n">
         <f aca="false">IF(B12="","",INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A12),$L$9:$L$38,0)))</f>
         <v>15</v>
       </c>
@@ -24534,40 +24584,44 @@
         <f aca="false">IF(B12="","",INDEX($K$9:$K$38,MATCH(LARGE($L$9:$L$38,A12),$L$9:$L$38,0)))</f>
         <v>1</v>
       </c>
-      <c r="E12" s="23" t="n">
+      <c r="E12" s="24" t="n">
         <f aca="false">IF(OR(B12="",$B$6=0),"",C12/$B$6)</f>
         <v>0.0588235294117647</v>
       </c>
-      <c r="F12" s="23" t="n">
+      <c r="F12" s="24" t="n">
         <f aca="false">IF(OR(B12="",$B$6=0),"",SUM($C$9:C12)/$B$6)</f>
         <v>0.941176470588235</v>
       </c>
-      <c r="I12" s="24" t="str">
+      <c r="I12" s="25" t="str">
         <f aca="false">IF(Setup!D8="","",IF(SUMPRODUCT(--(Setup!$D$4:D7=Setup!D8))&gt;0,"",Setup!D8))</f>
         <v>Changeover / setup</v>
       </c>
-      <c r="J12" s="24" t="n">
+      <c r="J12" s="25" t="n">
         <f aca="false">IF(I12="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I12)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0),'Downtime Log'!$G$5:$G$1004))</f>
         <v>65</v>
       </c>
-      <c r="K12" s="24" t="n">
+      <c r="K12" s="25" t="n">
         <f aca="false">IF(I12="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I12)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>2</v>
       </c>
-      <c r="L12" s="24" t="n">
+      <c r="L12" s="25" t="n">
         <f aca="false">IF(I12="",-1,J12+(34-4)/1000000)</f>
         <v>65.00003</v>
       </c>
+      <c r="M12" s="26" t="n">
+        <f aca="false">IF(B12&lt;&gt;"",F12,M11)</f>
+        <v>0.941176470588235</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="21" t="n">
+      <c r="A13" s="22" t="n">
         <v>5</v>
       </c>
       <c r="B13" s="10" t="str">
         <f aca="false">IF(INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A13),$L$9:$L$38,0))&lt;=0,"",INDEX($I$9:$I$38,MATCH(LARGE($L$9:$L$38,A13),$L$9:$L$38,0)))</f>
         <v>Quality hold / inspection</v>
       </c>
-      <c r="C13" s="22" t="n">
+      <c r="C13" s="23" t="n">
         <f aca="false">IF(B13="","",INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A13),$L$9:$L$38,0)))</f>
         <v>15</v>
       </c>
@@ -24575,40 +24629,44 @@
         <f aca="false">IF(B13="","",INDEX($K$9:$K$38,MATCH(LARGE($L$9:$L$38,A13),$L$9:$L$38,0)))</f>
         <v>1</v>
       </c>
-      <c r="E13" s="23" t="n">
+      <c r="E13" s="24" t="n">
         <f aca="false">IF(OR(B13="",$B$6=0),"",C13/$B$6)</f>
         <v>0.0588235294117647</v>
       </c>
-      <c r="F13" s="23" t="n">
+      <c r="F13" s="24" t="n">
         <f aca="false">IF(OR(B13="",$B$6=0),"",SUM($C$9:C13)/$B$6)</f>
         <v>1</v>
       </c>
-      <c r="I13" s="24" t="str">
+      <c r="I13" s="25" t="str">
         <f aca="false">IF(Setup!D9="","",IF(SUMPRODUCT(--(Setup!$D$4:D8=Setup!D9))&gt;0,"",Setup!D9))</f>
         <v>Adjustment / tuning</v>
       </c>
-      <c r="J13" s="24" t="n">
+      <c r="J13" s="25" t="n">
         <f aca="false">IF(I13="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I13)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0),'Downtime Log'!$G$5:$G$1004))</f>
         <v>0</v>
       </c>
-      <c r="K13" s="24" t="n">
+      <c r="K13" s="25" t="n">
         <f aca="false">IF(I13="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I13)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>0</v>
       </c>
-      <c r="L13" s="24" t="n">
+      <c r="L13" s="25" t="n">
         <f aca="false">IF(I13="",-1,J13+(34-5)/1000000)</f>
         <v>2.9E-005</v>
       </c>
+      <c r="M13" s="26" t="n">
+        <f aca="false">IF(B13&lt;&gt;"",F13,M12)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="21" t="n">
+      <c r="A14" s="22" t="n">
         <v>6</v>
       </c>
       <c r="B14" s="10" t="str">
         <f aca="false">IF(INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A14),$L$9:$L$38,0))&lt;=0,"",INDEX($I$9:$I$38,MATCH(LARGE($L$9:$L$38,A14),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="C14" s="22" t="str">
+      <c r="C14" s="23" t="str">
         <f aca="false">IF(B14="","",INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A14),$L$9:$L$38,0)))</f>
         <v/>
       </c>
@@ -24616,40 +24674,44 @@
         <f aca="false">IF(B14="","",INDEX($K$9:$K$38,MATCH(LARGE($L$9:$L$38,A14),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="E14" s="23" t="str">
+      <c r="E14" s="24" t="str">
         <f aca="false">IF(OR(B14="",$B$6=0),"",C14/$B$6)</f>
         <v/>
       </c>
-      <c r="F14" s="23" t="str">
+      <c r="F14" s="24" t="str">
         <f aca="false">IF(OR(B14="",$B$6=0),"",SUM($C$9:C14)/$B$6)</f>
         <v/>
       </c>
-      <c r="I14" s="24" t="str">
+      <c r="I14" s="25" t="str">
         <f aca="false">IF(Setup!D10="","",IF(SUMPRODUCT(--(Setup!$D$4:D9=Setup!D10))&gt;0,"",Setup!D10))</f>
         <v>Waiting for material</v>
       </c>
-      <c r="J14" s="24" t="n">
+      <c r="J14" s="25" t="n">
         <f aca="false">IF(I14="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I14)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0),'Downtime Log'!$G$5:$G$1004))</f>
         <v>15</v>
       </c>
-      <c r="K14" s="24" t="n">
+      <c r="K14" s="25" t="n">
         <f aca="false">IF(I14="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I14)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>1</v>
       </c>
-      <c r="L14" s="24" t="n">
+      <c r="L14" s="25" t="n">
         <f aca="false">IF(I14="",-1,J14+(34-6)/1000000)</f>
         <v>15.000028</v>
       </c>
+      <c r="M14" s="26" t="n">
+        <f aca="false">IF(B14&lt;&gt;"",F14,M13)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="21" t="n">
+      <c r="A15" s="22" t="n">
         <v>7</v>
       </c>
       <c r="B15" s="10" t="str">
         <f aca="false">IF(INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A15),$L$9:$L$38,0))&lt;=0,"",INDEX($I$9:$I$38,MATCH(LARGE($L$9:$L$38,A15),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="C15" s="22" t="str">
+      <c r="C15" s="23" t="str">
         <f aca="false">IF(B15="","",INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A15),$L$9:$L$38,0)))</f>
         <v/>
       </c>
@@ -24657,40 +24719,44 @@
         <f aca="false">IF(B15="","",INDEX($K$9:$K$38,MATCH(LARGE($L$9:$L$38,A15),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="E15" s="23" t="str">
+      <c r="E15" s="24" t="str">
         <f aca="false">IF(OR(B15="",$B$6=0),"",C15/$B$6)</f>
         <v/>
       </c>
-      <c r="F15" s="23" t="str">
+      <c r="F15" s="24" t="str">
         <f aca="false">IF(OR(B15="",$B$6=0),"",SUM($C$9:C15)/$B$6)</f>
         <v/>
       </c>
-      <c r="I15" s="24" t="str">
+      <c r="I15" s="25" t="str">
         <f aca="false">IF(Setup!D11="","",IF(SUMPRODUCT(--(Setup!$D$4:D10=Setup!D11))&gt;0,"",Setup!D11))</f>
         <v>Waiting for upstream process</v>
       </c>
-      <c r="J15" s="24" t="n">
+      <c r="J15" s="25" t="n">
         <f aca="false">IF(I15="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I15)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0),'Downtime Log'!$G$5:$G$1004))</f>
         <v>0</v>
       </c>
-      <c r="K15" s="24" t="n">
+      <c r="K15" s="25" t="n">
         <f aca="false">IF(I15="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I15)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>0</v>
       </c>
-      <c r="L15" s="24" t="n">
+      <c r="L15" s="25" t="n">
         <f aca="false">IF(I15="",-1,J15+(34-7)/1000000)</f>
         <v>2.7E-005</v>
       </c>
+      <c r="M15" s="26" t="n">
+        <f aca="false">IF(B15&lt;&gt;"",F15,M14)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="21" t="n">
+      <c r="A16" s="22" t="n">
         <v>8</v>
       </c>
       <c r="B16" s="10" t="str">
         <f aca="false">IF(INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A16),$L$9:$L$38,0))&lt;=0,"",INDEX($I$9:$I$38,MATCH(LARGE($L$9:$L$38,A16),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="C16" s="22" t="str">
+      <c r="C16" s="23" t="str">
         <f aca="false">IF(B16="","",INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A16),$L$9:$L$38,0)))</f>
         <v/>
       </c>
@@ -24698,40 +24764,44 @@
         <f aca="false">IF(B16="","",INDEX($K$9:$K$38,MATCH(LARGE($L$9:$L$38,A16),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="E16" s="23" t="str">
+      <c r="E16" s="24" t="str">
         <f aca="false">IF(OR(B16="",$B$6=0),"",C16/$B$6)</f>
         <v/>
       </c>
-      <c r="F16" s="23" t="str">
+      <c r="F16" s="24" t="str">
         <f aca="false">IF(OR(B16="",$B$6=0),"",SUM($C$9:C16)/$B$6)</f>
         <v/>
       </c>
-      <c r="I16" s="24" t="str">
+      <c r="I16" s="25" t="str">
         <f aca="false">IF(Setup!D12="","",IF(SUMPRODUCT(--(Setup!$D$4:D11=Setup!D12))&gt;0,"",Setup!D12))</f>
         <v>Quality hold / inspection</v>
       </c>
-      <c r="J16" s="24" t="n">
+      <c r="J16" s="25" t="n">
         <f aca="false">IF(I16="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I16)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0),'Downtime Log'!$G$5:$G$1004))</f>
         <v>15</v>
       </c>
-      <c r="K16" s="24" t="n">
+      <c r="K16" s="25" t="n">
         <f aca="false">IF(I16="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I16)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>1</v>
       </c>
-      <c r="L16" s="24" t="n">
+      <c r="L16" s="25" t="n">
         <f aca="false">IF(I16="",-1,J16+(34-8)/1000000)</f>
         <v>15.000026</v>
       </c>
+      <c r="M16" s="26" t="n">
+        <f aca="false">IF(B16&lt;&gt;"",F16,M15)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="21" t="n">
+      <c r="A17" s="22" t="n">
         <v>9</v>
       </c>
       <c r="B17" s="10" t="str">
         <f aca="false">IF(INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A17),$L$9:$L$38,0))&lt;=0,"",INDEX($I$9:$I$38,MATCH(LARGE($L$9:$L$38,A17),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="C17" s="22" t="str">
+      <c r="C17" s="23" t="str">
         <f aca="false">IF(B17="","",INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A17),$L$9:$L$38,0)))</f>
         <v/>
       </c>
@@ -24739,40 +24809,44 @@
         <f aca="false">IF(B17="","",INDEX($K$9:$K$38,MATCH(LARGE($L$9:$L$38,A17),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="E17" s="23" t="str">
+      <c r="E17" s="24" t="str">
         <f aca="false">IF(OR(B17="",$B$6=0),"",C17/$B$6)</f>
         <v/>
       </c>
-      <c r="F17" s="23" t="str">
+      <c r="F17" s="24" t="str">
         <f aca="false">IF(OR(B17="",$B$6=0),"",SUM($C$9:C17)/$B$6)</f>
         <v/>
       </c>
-      <c r="I17" s="24" t="str">
+      <c r="I17" s="25" t="str">
         <f aca="false">IF(Setup!D13="","",IF(SUMPRODUCT(--(Setup!$D$4:D12=Setup!D13))&gt;0,"",Setup!D13))</f>
         <v>No operator available</v>
       </c>
-      <c r="J17" s="24" t="n">
+      <c r="J17" s="25" t="n">
         <f aca="false">IF(I17="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I17)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0),'Downtime Log'!$G$5:$G$1004))</f>
         <v>0</v>
       </c>
-      <c r="K17" s="24" t="n">
+      <c r="K17" s="25" t="n">
         <f aca="false">IF(I17="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I17)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>0</v>
       </c>
-      <c r="L17" s="24" t="n">
+      <c r="L17" s="25" t="n">
         <f aca="false">IF(I17="",-1,J17+(34-9)/1000000)</f>
         <v>2.5E-005</v>
       </c>
+      <c r="M17" s="26" t="n">
+        <f aca="false">IF(B17&lt;&gt;"",F17,M16)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="21" t="n">
+      <c r="A18" s="22" t="n">
         <v>10</v>
       </c>
       <c r="B18" s="10" t="str">
         <f aca="false">IF(INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A18),$L$9:$L$38,0))&lt;=0,"",INDEX($I$9:$I$38,MATCH(LARGE($L$9:$L$38,A18),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="C18" s="22" t="str">
+      <c r="C18" s="23" t="str">
         <f aca="false">IF(B18="","",INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A18),$L$9:$L$38,0)))</f>
         <v/>
       </c>
@@ -24780,40 +24854,44 @@
         <f aca="false">IF(B18="","",INDEX($K$9:$K$38,MATCH(LARGE($L$9:$L$38,A18),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="E18" s="23" t="str">
+      <c r="E18" s="24" t="str">
         <f aca="false">IF(OR(B18="",$B$6=0),"",C18/$B$6)</f>
         <v/>
       </c>
-      <c r="F18" s="23" t="str">
+      <c r="F18" s="24" t="str">
         <f aca="false">IF(OR(B18="",$B$6=0),"",SUM($C$9:C18)/$B$6)</f>
         <v/>
       </c>
-      <c r="I18" s="24" t="str">
+      <c r="I18" s="25" t="str">
         <f aca="false">IF(Setup!D14="","",IF(SUMPRODUCT(--(Setup!$D$4:D13=Setup!D14))&gt;0,"",Setup!D14))</f>
         <v>Planned maintenance</v>
       </c>
-      <c r="J18" s="24" t="n">
+      <c r="J18" s="25" t="n">
         <f aca="false">IF(I18="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I18)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0),'Downtime Log'!$G$5:$G$1004))</f>
         <v>0</v>
       </c>
-      <c r="K18" s="24" t="n">
+      <c r="K18" s="25" t="n">
         <f aca="false">IF(I18="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I18)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>0</v>
       </c>
-      <c r="L18" s="24" t="n">
+      <c r="L18" s="25" t="n">
         <f aca="false">IF(I18="",-1,J18+(34-10)/1000000)</f>
         <v>2.4E-005</v>
       </c>
+      <c r="M18" s="26" t="n">
+        <f aca="false">IF(B18&lt;&gt;"",F18,M17)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="21" t="n">
+      <c r="A19" s="22" t="n">
         <v>11</v>
       </c>
       <c r="B19" s="10" t="str">
         <f aca="false">IF(INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A19),$L$9:$L$38,0))&lt;=0,"",INDEX($I$9:$I$38,MATCH(LARGE($L$9:$L$38,A19),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="C19" s="22" t="str">
+      <c r="C19" s="23" t="str">
         <f aca="false">IF(B19="","",INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A19),$L$9:$L$38,0)))</f>
         <v/>
       </c>
@@ -24821,40 +24899,44 @@
         <f aca="false">IF(B19="","",INDEX($K$9:$K$38,MATCH(LARGE($L$9:$L$38,A19),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="E19" s="23" t="str">
+      <c r="E19" s="24" t="str">
         <f aca="false">IF(OR(B19="",$B$6=0),"",C19/$B$6)</f>
         <v/>
       </c>
-      <c r="F19" s="23" t="str">
+      <c r="F19" s="24" t="str">
         <f aca="false">IF(OR(B19="",$B$6=0),"",SUM($C$9:C19)/$B$6)</f>
         <v/>
       </c>
-      <c r="I19" s="24" t="str">
+      <c r="I19" s="25" t="str">
         <f aca="false">IF(Setup!D15="","",IF(SUMPRODUCT(--(Setup!$D$4:D14=Setup!D15))&gt;0,"",Setup!D15))</f>
         <v>Meeting / training</v>
       </c>
-      <c r="J19" s="24" t="n">
+      <c r="J19" s="25" t="n">
         <f aca="false">IF(I19="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I19)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0),'Downtime Log'!$G$5:$G$1004))</f>
         <v>0</v>
       </c>
-      <c r="K19" s="24" t="n">
+      <c r="K19" s="25" t="n">
         <f aca="false">IF(I19="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I19)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>0</v>
       </c>
-      <c r="L19" s="24" t="n">
+      <c r="L19" s="25" t="n">
         <f aca="false">IF(I19="",-1,J19+(34-11)/1000000)</f>
         <v>2.3E-005</v>
       </c>
+      <c r="M19" s="26" t="n">
+        <f aca="false">IF(B19&lt;&gt;"",F19,M18)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="21" t="n">
+      <c r="A20" s="22" t="n">
         <v>12</v>
       </c>
       <c r="B20" s="10" t="str">
         <f aca="false">IF(INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A20),$L$9:$L$38,0))&lt;=0,"",INDEX($I$9:$I$38,MATCH(LARGE($L$9:$L$38,A20),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="C20" s="22" t="str">
+      <c r="C20" s="23" t="str">
         <f aca="false">IF(B20="","",INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A20),$L$9:$L$38,0)))</f>
         <v/>
       </c>
@@ -24862,40 +24944,44 @@
         <f aca="false">IF(B20="","",INDEX($K$9:$K$38,MATCH(LARGE($L$9:$L$38,A20),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="E20" s="23" t="str">
+      <c r="E20" s="24" t="str">
         <f aca="false">IF(OR(B20="",$B$6=0),"",C20/$B$6)</f>
         <v/>
       </c>
-      <c r="F20" s="23" t="str">
+      <c r="F20" s="24" t="str">
         <f aca="false">IF(OR(B20="",$B$6=0),"",SUM($C$9:C20)/$B$6)</f>
         <v/>
       </c>
-      <c r="I20" s="24" t="str">
+      <c r="I20" s="25" t="str">
         <f aca="false">IF(Setup!D16="","",IF(SUMPRODUCT(--(Setup!$D$4:D15=Setup!D16))&gt;0,"",Setup!D16))</f>
         <v>Other (describe in notes)</v>
       </c>
-      <c r="J20" s="24" t="n">
+      <c r="J20" s="25" t="n">
         <f aca="false">IF(I20="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I20)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0),'Downtime Log'!$G$5:$G$1004))</f>
         <v>0</v>
       </c>
-      <c r="K20" s="24" t="n">
+      <c r="K20" s="25" t="n">
         <f aca="false">IF(I20="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I20)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>0</v>
       </c>
-      <c r="L20" s="24" t="n">
+      <c r="L20" s="25" t="n">
         <f aca="false">IF(I20="",-1,J20+(34-12)/1000000)</f>
         <v>2.2E-005</v>
       </c>
+      <c r="M20" s="26" t="n">
+        <f aca="false">IF(B20&lt;&gt;"",F20,M19)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="21" t="n">
+      <c r="A21" s="22" t="n">
         <v>13</v>
       </c>
       <c r="B21" s="10" t="str">
         <f aca="false">IF(INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A21),$L$9:$L$38,0))&lt;=0,"",INDEX($I$9:$I$38,MATCH(LARGE($L$9:$L$38,A21),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="C21" s="22" t="str">
+      <c r="C21" s="23" t="str">
         <f aca="false">IF(B21="","",INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A21),$L$9:$L$38,0)))</f>
         <v/>
       </c>
@@ -24903,40 +24989,44 @@
         <f aca="false">IF(B21="","",INDEX($K$9:$K$38,MATCH(LARGE($L$9:$L$38,A21),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="E21" s="23" t="str">
+      <c r="E21" s="24" t="str">
         <f aca="false">IF(OR(B21="",$B$6=0),"",C21/$B$6)</f>
         <v/>
       </c>
-      <c r="F21" s="23" t="str">
+      <c r="F21" s="24" t="str">
         <f aca="false">IF(OR(B21="",$B$6=0),"",SUM($C$9:C21)/$B$6)</f>
         <v/>
       </c>
-      <c r="I21" s="24" t="str">
+      <c r="I21" s="25" t="str">
         <f aca="false">IF(Setup!D17="","",IF(SUMPRODUCT(--(Setup!$D$4:D16=Setup!D17))&gt;0,"",Setup!D17))</f>
         <v/>
       </c>
-      <c r="J21" s="24" t="n">
+      <c r="J21" s="25" t="n">
         <f aca="false">IF(I21="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I21)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0),'Downtime Log'!$G$5:$G$1004))</f>
         <v>0</v>
       </c>
-      <c r="K21" s="24" t="n">
+      <c r="K21" s="25" t="n">
         <f aca="false">IF(I21="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I21)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>0</v>
       </c>
-      <c r="L21" s="24" t="n">
+      <c r="L21" s="25" t="n">
         <f aca="false">IF(I21="",-1,J21+(34-13)/1000000)</f>
         <v>-1</v>
       </c>
+      <c r="M21" s="26" t="n">
+        <f aca="false">IF(B21&lt;&gt;"",F21,M20)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="21" t="n">
+      <c r="A22" s="22" t="n">
         <v>14</v>
       </c>
       <c r="B22" s="10" t="str">
         <f aca="false">IF(INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A22),$L$9:$L$38,0))&lt;=0,"",INDEX($I$9:$I$38,MATCH(LARGE($L$9:$L$38,A22),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="C22" s="22" t="str">
+      <c r="C22" s="23" t="str">
         <f aca="false">IF(B22="","",INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A22),$L$9:$L$38,0)))</f>
         <v/>
       </c>
@@ -24944,40 +25034,44 @@
         <f aca="false">IF(B22="","",INDEX($K$9:$K$38,MATCH(LARGE($L$9:$L$38,A22),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="E22" s="23" t="str">
+      <c r="E22" s="24" t="str">
         <f aca="false">IF(OR(B22="",$B$6=0),"",C22/$B$6)</f>
         <v/>
       </c>
-      <c r="F22" s="23" t="str">
+      <c r="F22" s="24" t="str">
         <f aca="false">IF(OR(B22="",$B$6=0),"",SUM($C$9:C22)/$B$6)</f>
         <v/>
       </c>
-      <c r="I22" s="24" t="str">
+      <c r="I22" s="25" t="str">
         <f aca="false">IF(Setup!D18="","",IF(SUMPRODUCT(--(Setup!$D$4:D17=Setup!D18))&gt;0,"",Setup!D18))</f>
         <v/>
       </c>
-      <c r="J22" s="24" t="n">
+      <c r="J22" s="25" t="n">
         <f aca="false">IF(I22="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I22)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0),'Downtime Log'!$G$5:$G$1004))</f>
         <v>0</v>
       </c>
-      <c r="K22" s="24" t="n">
+      <c r="K22" s="25" t="n">
         <f aca="false">IF(I22="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I22)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>0</v>
       </c>
-      <c r="L22" s="24" t="n">
+      <c r="L22" s="25" t="n">
         <f aca="false">IF(I22="",-1,J22+(34-14)/1000000)</f>
         <v>-1</v>
       </c>
+      <c r="M22" s="26" t="n">
+        <f aca="false">IF(B22&lt;&gt;"",F22,M21)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="21" t="n">
+      <c r="A23" s="22" t="n">
         <v>15</v>
       </c>
       <c r="B23" s="10" t="str">
         <f aca="false">IF(INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A23),$L$9:$L$38,0))&lt;=0,"",INDEX($I$9:$I$38,MATCH(LARGE($L$9:$L$38,A23),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="C23" s="22" t="str">
+      <c r="C23" s="23" t="str">
         <f aca="false">IF(B23="","",INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A23),$L$9:$L$38,0)))</f>
         <v/>
       </c>
@@ -24985,40 +25079,44 @@
         <f aca="false">IF(B23="","",INDEX($K$9:$K$38,MATCH(LARGE($L$9:$L$38,A23),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="E23" s="23" t="str">
+      <c r="E23" s="24" t="str">
         <f aca="false">IF(OR(B23="",$B$6=0),"",C23/$B$6)</f>
         <v/>
       </c>
-      <c r="F23" s="23" t="str">
+      <c r="F23" s="24" t="str">
         <f aca="false">IF(OR(B23="",$B$6=0),"",SUM($C$9:C23)/$B$6)</f>
         <v/>
       </c>
-      <c r="I23" s="24" t="str">
+      <c r="I23" s="25" t="str">
         <f aca="false">IF(Setup!D19="","",IF(SUMPRODUCT(--(Setup!$D$4:D18=Setup!D19))&gt;0,"",Setup!D19))</f>
         <v/>
       </c>
-      <c r="J23" s="24" t="n">
+      <c r="J23" s="25" t="n">
         <f aca="false">IF(I23="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I23)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0),'Downtime Log'!$G$5:$G$1004))</f>
         <v>0</v>
       </c>
-      <c r="K23" s="24" t="n">
+      <c r="K23" s="25" t="n">
         <f aca="false">IF(I23="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I23)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>0</v>
       </c>
-      <c r="L23" s="24" t="n">
+      <c r="L23" s="25" t="n">
         <f aca="false">IF(I23="",-1,J23+(34-15)/1000000)</f>
         <v>-1</v>
       </c>
+      <c r="M23" s="26" t="n">
+        <f aca="false">IF(B23&lt;&gt;"",F23,M22)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="21" t="n">
+      <c r="A24" s="22" t="n">
         <v>16</v>
       </c>
       <c r="B24" s="10" t="str">
         <f aca="false">IF(INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A24),$L$9:$L$38,0))&lt;=0,"",INDEX($I$9:$I$38,MATCH(LARGE($L$9:$L$38,A24),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="C24" s="22" t="str">
+      <c r="C24" s="23" t="str">
         <f aca="false">IF(B24="","",INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A24),$L$9:$L$38,0)))</f>
         <v/>
       </c>
@@ -25026,40 +25124,44 @@
         <f aca="false">IF(B24="","",INDEX($K$9:$K$38,MATCH(LARGE($L$9:$L$38,A24),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="E24" s="23" t="str">
+      <c r="E24" s="24" t="str">
         <f aca="false">IF(OR(B24="",$B$6=0),"",C24/$B$6)</f>
         <v/>
       </c>
-      <c r="F24" s="23" t="str">
+      <c r="F24" s="24" t="str">
         <f aca="false">IF(OR(B24="",$B$6=0),"",SUM($C$9:C24)/$B$6)</f>
         <v/>
       </c>
-      <c r="I24" s="24" t="str">
+      <c r="I24" s="25" t="str">
         <f aca="false">IF(Setup!D20="","",IF(SUMPRODUCT(--(Setup!$D$4:D19=Setup!D20))&gt;0,"",Setup!D20))</f>
         <v/>
       </c>
-      <c r="J24" s="24" t="n">
+      <c r="J24" s="25" t="n">
         <f aca="false">IF(I24="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I24)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0),'Downtime Log'!$G$5:$G$1004))</f>
         <v>0</v>
       </c>
-      <c r="K24" s="24" t="n">
+      <c r="K24" s="25" t="n">
         <f aca="false">IF(I24="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I24)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>0</v>
       </c>
-      <c r="L24" s="24" t="n">
+      <c r="L24" s="25" t="n">
         <f aca="false">IF(I24="",-1,J24+(34-16)/1000000)</f>
         <v>-1</v>
       </c>
+      <c r="M24" s="26" t="n">
+        <f aca="false">IF(B24&lt;&gt;"",F24,M23)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="21" t="n">
+      <c r="A25" s="22" t="n">
         <v>17</v>
       </c>
       <c r="B25" s="10" t="str">
         <f aca="false">IF(INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A25),$L$9:$L$38,0))&lt;=0,"",INDEX($I$9:$I$38,MATCH(LARGE($L$9:$L$38,A25),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="C25" s="22" t="str">
+      <c r="C25" s="23" t="str">
         <f aca="false">IF(B25="","",INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A25),$L$9:$L$38,0)))</f>
         <v/>
       </c>
@@ -25067,40 +25169,44 @@
         <f aca="false">IF(B25="","",INDEX($K$9:$K$38,MATCH(LARGE($L$9:$L$38,A25),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="E25" s="23" t="str">
+      <c r="E25" s="24" t="str">
         <f aca="false">IF(OR(B25="",$B$6=0),"",C25/$B$6)</f>
         <v/>
       </c>
-      <c r="F25" s="23" t="str">
+      <c r="F25" s="24" t="str">
         <f aca="false">IF(OR(B25="",$B$6=0),"",SUM($C$9:C25)/$B$6)</f>
         <v/>
       </c>
-      <c r="I25" s="24" t="str">
+      <c r="I25" s="25" t="str">
         <f aca="false">IF(Setup!D21="","",IF(SUMPRODUCT(--(Setup!$D$4:D20=Setup!D21))&gt;0,"",Setup!D21))</f>
         <v/>
       </c>
-      <c r="J25" s="24" t="n">
+      <c r="J25" s="25" t="n">
         <f aca="false">IF(I25="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I25)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0),'Downtime Log'!$G$5:$G$1004))</f>
         <v>0</v>
       </c>
-      <c r="K25" s="24" t="n">
+      <c r="K25" s="25" t="n">
         <f aca="false">IF(I25="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I25)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>0</v>
       </c>
-      <c r="L25" s="24" t="n">
+      <c r="L25" s="25" t="n">
         <f aca="false">IF(I25="",-1,J25+(34-17)/1000000)</f>
         <v>-1</v>
       </c>
+      <c r="M25" s="26" t="n">
+        <f aca="false">IF(B25&lt;&gt;"",F25,M24)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="21" t="n">
+      <c r="A26" s="22" t="n">
         <v>18</v>
       </c>
       <c r="B26" s="10" t="str">
         <f aca="false">IF(INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A26),$L$9:$L$38,0))&lt;=0,"",INDEX($I$9:$I$38,MATCH(LARGE($L$9:$L$38,A26),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="C26" s="22" t="str">
+      <c r="C26" s="23" t="str">
         <f aca="false">IF(B26="","",INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A26),$L$9:$L$38,0)))</f>
         <v/>
       </c>
@@ -25108,40 +25214,44 @@
         <f aca="false">IF(B26="","",INDEX($K$9:$K$38,MATCH(LARGE($L$9:$L$38,A26),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="E26" s="23" t="str">
+      <c r="E26" s="24" t="str">
         <f aca="false">IF(OR(B26="",$B$6=0),"",C26/$B$6)</f>
         <v/>
       </c>
-      <c r="F26" s="23" t="str">
+      <c r="F26" s="24" t="str">
         <f aca="false">IF(OR(B26="",$B$6=0),"",SUM($C$9:C26)/$B$6)</f>
         <v/>
       </c>
-      <c r="I26" s="24" t="str">
+      <c r="I26" s="25" t="str">
         <f aca="false">IF(Setup!D22="","",IF(SUMPRODUCT(--(Setup!$D$4:D21=Setup!D22))&gt;0,"",Setup!D22))</f>
         <v/>
       </c>
-      <c r="J26" s="24" t="n">
+      <c r="J26" s="25" t="n">
         <f aca="false">IF(I26="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I26)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0),'Downtime Log'!$G$5:$G$1004))</f>
         <v>0</v>
       </c>
-      <c r="K26" s="24" t="n">
+      <c r="K26" s="25" t="n">
         <f aca="false">IF(I26="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I26)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>0</v>
       </c>
-      <c r="L26" s="24" t="n">
+      <c r="L26" s="25" t="n">
         <f aca="false">IF(I26="",-1,J26+(34-18)/1000000)</f>
         <v>-1</v>
       </c>
+      <c r="M26" s="26" t="n">
+        <f aca="false">IF(B26&lt;&gt;"",F26,M25)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="21" t="n">
+      <c r="A27" s="22" t="n">
         <v>19</v>
       </c>
       <c r="B27" s="10" t="str">
         <f aca="false">IF(INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A27),$L$9:$L$38,0))&lt;=0,"",INDEX($I$9:$I$38,MATCH(LARGE($L$9:$L$38,A27),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="C27" s="22" t="str">
+      <c r="C27" s="23" t="str">
         <f aca="false">IF(B27="","",INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A27),$L$9:$L$38,0)))</f>
         <v/>
       </c>
@@ -25149,40 +25259,44 @@
         <f aca="false">IF(B27="","",INDEX($K$9:$K$38,MATCH(LARGE($L$9:$L$38,A27),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="E27" s="23" t="str">
+      <c r="E27" s="24" t="str">
         <f aca="false">IF(OR(B27="",$B$6=0),"",C27/$B$6)</f>
         <v/>
       </c>
-      <c r="F27" s="23" t="str">
+      <c r="F27" s="24" t="str">
         <f aca="false">IF(OR(B27="",$B$6=0),"",SUM($C$9:C27)/$B$6)</f>
         <v/>
       </c>
-      <c r="I27" s="24" t="str">
+      <c r="I27" s="25" t="str">
         <f aca="false">IF(Setup!D23="","",IF(SUMPRODUCT(--(Setup!$D$4:D22=Setup!D23))&gt;0,"",Setup!D23))</f>
         <v/>
       </c>
-      <c r="J27" s="24" t="n">
+      <c r="J27" s="25" t="n">
         <f aca="false">IF(I27="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I27)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0),'Downtime Log'!$G$5:$G$1004))</f>
         <v>0</v>
       </c>
-      <c r="K27" s="24" t="n">
+      <c r="K27" s="25" t="n">
         <f aca="false">IF(I27="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I27)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>0</v>
       </c>
-      <c r="L27" s="24" t="n">
+      <c r="L27" s="25" t="n">
         <f aca="false">IF(I27="",-1,J27+(34-19)/1000000)</f>
         <v>-1</v>
       </c>
+      <c r="M27" s="26" t="n">
+        <f aca="false">IF(B27&lt;&gt;"",F27,M26)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="21" t="n">
+      <c r="A28" s="22" t="n">
         <v>20</v>
       </c>
       <c r="B28" s="10" t="str">
         <f aca="false">IF(INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A28),$L$9:$L$38,0))&lt;=0,"",INDEX($I$9:$I$38,MATCH(LARGE($L$9:$L$38,A28),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="C28" s="22" t="str">
+      <c r="C28" s="23" t="str">
         <f aca="false">IF(B28="","",INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A28),$L$9:$L$38,0)))</f>
         <v/>
       </c>
@@ -25190,40 +25304,44 @@
         <f aca="false">IF(B28="","",INDEX($K$9:$K$38,MATCH(LARGE($L$9:$L$38,A28),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="E28" s="23" t="str">
+      <c r="E28" s="24" t="str">
         <f aca="false">IF(OR(B28="",$B$6=0),"",C28/$B$6)</f>
         <v/>
       </c>
-      <c r="F28" s="23" t="str">
+      <c r="F28" s="24" t="str">
         <f aca="false">IF(OR(B28="",$B$6=0),"",SUM($C$9:C28)/$B$6)</f>
         <v/>
       </c>
-      <c r="I28" s="24" t="str">
+      <c r="I28" s="25" t="str">
         <f aca="false">IF(Setup!D24="","",IF(SUMPRODUCT(--(Setup!$D$4:D23=Setup!D24))&gt;0,"",Setup!D24))</f>
         <v/>
       </c>
-      <c r="J28" s="24" t="n">
+      <c r="J28" s="25" t="n">
         <f aca="false">IF(I28="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I28)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0),'Downtime Log'!$G$5:$G$1004))</f>
         <v>0</v>
       </c>
-      <c r="K28" s="24" t="n">
+      <c r="K28" s="25" t="n">
         <f aca="false">IF(I28="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I28)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>0</v>
       </c>
-      <c r="L28" s="24" t="n">
+      <c r="L28" s="25" t="n">
         <f aca="false">IF(I28="",-1,J28+(34-20)/1000000)</f>
         <v>-1</v>
       </c>
+      <c r="M28" s="26" t="n">
+        <f aca="false">IF(B28&lt;&gt;"",F28,M27)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="21" t="n">
+      <c r="A29" s="22" t="n">
         <v>21</v>
       </c>
       <c r="B29" s="10" t="str">
         <f aca="false">IF(INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A29),$L$9:$L$38,0))&lt;=0,"",INDEX($I$9:$I$38,MATCH(LARGE($L$9:$L$38,A29),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="C29" s="22" t="str">
+      <c r="C29" s="23" t="str">
         <f aca="false">IF(B29="","",INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A29),$L$9:$L$38,0)))</f>
         <v/>
       </c>
@@ -25231,40 +25349,44 @@
         <f aca="false">IF(B29="","",INDEX($K$9:$K$38,MATCH(LARGE($L$9:$L$38,A29),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="E29" s="23" t="str">
+      <c r="E29" s="24" t="str">
         <f aca="false">IF(OR(B29="",$B$6=0),"",C29/$B$6)</f>
         <v/>
       </c>
-      <c r="F29" s="23" t="str">
+      <c r="F29" s="24" t="str">
         <f aca="false">IF(OR(B29="",$B$6=0),"",SUM($C$9:C29)/$B$6)</f>
         <v/>
       </c>
-      <c r="I29" s="24" t="str">
+      <c r="I29" s="25" t="str">
         <f aca="false">IF(Setup!D25="","",IF(SUMPRODUCT(--(Setup!$D$4:D24=Setup!D25))&gt;0,"",Setup!D25))</f>
         <v/>
       </c>
-      <c r="J29" s="24" t="n">
+      <c r="J29" s="25" t="n">
         <f aca="false">IF(I29="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I29)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0),'Downtime Log'!$G$5:$G$1004))</f>
         <v>0</v>
       </c>
-      <c r="K29" s="24" t="n">
+      <c r="K29" s="25" t="n">
         <f aca="false">IF(I29="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I29)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>0</v>
       </c>
-      <c r="L29" s="24" t="n">
+      <c r="L29" s="25" t="n">
         <f aca="false">IF(I29="",-1,J29+(34-21)/1000000)</f>
         <v>-1</v>
       </c>
+      <c r="M29" s="26" t="n">
+        <f aca="false">IF(B29&lt;&gt;"",F29,M28)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="21" t="n">
+      <c r="A30" s="22" t="n">
         <v>22</v>
       </c>
       <c r="B30" s="10" t="str">
         <f aca="false">IF(INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A30),$L$9:$L$38,0))&lt;=0,"",INDEX($I$9:$I$38,MATCH(LARGE($L$9:$L$38,A30),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="C30" s="22" t="str">
+      <c r="C30" s="23" t="str">
         <f aca="false">IF(B30="","",INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A30),$L$9:$L$38,0)))</f>
         <v/>
       </c>
@@ -25272,40 +25394,44 @@
         <f aca="false">IF(B30="","",INDEX($K$9:$K$38,MATCH(LARGE($L$9:$L$38,A30),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="E30" s="23" t="str">
+      <c r="E30" s="24" t="str">
         <f aca="false">IF(OR(B30="",$B$6=0),"",C30/$B$6)</f>
         <v/>
       </c>
-      <c r="F30" s="23" t="str">
+      <c r="F30" s="24" t="str">
         <f aca="false">IF(OR(B30="",$B$6=0),"",SUM($C$9:C30)/$B$6)</f>
         <v/>
       </c>
-      <c r="I30" s="24" t="str">
+      <c r="I30" s="25" t="str">
         <f aca="false">IF(Setup!D26="","",IF(SUMPRODUCT(--(Setup!$D$4:D25=Setup!D26))&gt;0,"",Setup!D26))</f>
         <v/>
       </c>
-      <c r="J30" s="24" t="n">
+      <c r="J30" s="25" t="n">
         <f aca="false">IF(I30="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I30)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0),'Downtime Log'!$G$5:$G$1004))</f>
         <v>0</v>
       </c>
-      <c r="K30" s="24" t="n">
+      <c r="K30" s="25" t="n">
         <f aca="false">IF(I30="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I30)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>0</v>
       </c>
-      <c r="L30" s="24" t="n">
+      <c r="L30" s="25" t="n">
         <f aca="false">IF(I30="",-1,J30+(34-22)/1000000)</f>
         <v>-1</v>
       </c>
+      <c r="M30" s="26" t="n">
+        <f aca="false">IF(B30&lt;&gt;"",F30,M29)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="21" t="n">
+      <c r="A31" s="22" t="n">
         <v>23</v>
       </c>
       <c r="B31" s="10" t="str">
         <f aca="false">IF(INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A31),$L$9:$L$38,0))&lt;=0,"",INDEX($I$9:$I$38,MATCH(LARGE($L$9:$L$38,A31),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="C31" s="22" t="str">
+      <c r="C31" s="23" t="str">
         <f aca="false">IF(B31="","",INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A31),$L$9:$L$38,0)))</f>
         <v/>
       </c>
@@ -25313,40 +25439,44 @@
         <f aca="false">IF(B31="","",INDEX($K$9:$K$38,MATCH(LARGE($L$9:$L$38,A31),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="E31" s="23" t="str">
+      <c r="E31" s="24" t="str">
         <f aca="false">IF(OR(B31="",$B$6=0),"",C31/$B$6)</f>
         <v/>
       </c>
-      <c r="F31" s="23" t="str">
+      <c r="F31" s="24" t="str">
         <f aca="false">IF(OR(B31="",$B$6=0),"",SUM($C$9:C31)/$B$6)</f>
         <v/>
       </c>
-      <c r="I31" s="24" t="str">
+      <c r="I31" s="25" t="str">
         <f aca="false">IF(Setup!D27="","",IF(SUMPRODUCT(--(Setup!$D$4:D26=Setup!D27))&gt;0,"",Setup!D27))</f>
         <v/>
       </c>
-      <c r="J31" s="24" t="n">
+      <c r="J31" s="25" t="n">
         <f aca="false">IF(I31="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I31)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0),'Downtime Log'!$G$5:$G$1004))</f>
         <v>0</v>
       </c>
-      <c r="K31" s="24" t="n">
+      <c r="K31" s="25" t="n">
         <f aca="false">IF(I31="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I31)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>0</v>
       </c>
-      <c r="L31" s="24" t="n">
+      <c r="L31" s="25" t="n">
         <f aca="false">IF(I31="",-1,J31+(34-23)/1000000)</f>
         <v>-1</v>
       </c>
+      <c r="M31" s="26" t="n">
+        <f aca="false">IF(B31&lt;&gt;"",F31,M30)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="21" t="n">
+      <c r="A32" s="22" t="n">
         <v>24</v>
       </c>
       <c r="B32" s="10" t="str">
         <f aca="false">IF(INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A32),$L$9:$L$38,0))&lt;=0,"",INDEX($I$9:$I$38,MATCH(LARGE($L$9:$L$38,A32),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="C32" s="22" t="str">
+      <c r="C32" s="23" t="str">
         <f aca="false">IF(B32="","",INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A32),$L$9:$L$38,0)))</f>
         <v/>
       </c>
@@ -25354,40 +25484,44 @@
         <f aca="false">IF(B32="","",INDEX($K$9:$K$38,MATCH(LARGE($L$9:$L$38,A32),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="E32" s="23" t="str">
+      <c r="E32" s="24" t="str">
         <f aca="false">IF(OR(B32="",$B$6=0),"",C32/$B$6)</f>
         <v/>
       </c>
-      <c r="F32" s="23" t="str">
+      <c r="F32" s="24" t="str">
         <f aca="false">IF(OR(B32="",$B$6=0),"",SUM($C$9:C32)/$B$6)</f>
         <v/>
       </c>
-      <c r="I32" s="24" t="str">
+      <c r="I32" s="25" t="str">
         <f aca="false">IF(Setup!D28="","",IF(SUMPRODUCT(--(Setup!$D$4:D27=Setup!D28))&gt;0,"",Setup!D28))</f>
         <v/>
       </c>
-      <c r="J32" s="24" t="n">
+      <c r="J32" s="25" t="n">
         <f aca="false">IF(I32="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I32)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0),'Downtime Log'!$G$5:$G$1004))</f>
         <v>0</v>
       </c>
-      <c r="K32" s="24" t="n">
+      <c r="K32" s="25" t="n">
         <f aca="false">IF(I32="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I32)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>0</v>
       </c>
-      <c r="L32" s="24" t="n">
+      <c r="L32" s="25" t="n">
         <f aca="false">IF(I32="",-1,J32+(34-24)/1000000)</f>
         <v>-1</v>
       </c>
+      <c r="M32" s="26" t="n">
+        <f aca="false">IF(B32&lt;&gt;"",F32,M31)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="21" t="n">
+      <c r="A33" s="22" t="n">
         <v>25</v>
       </c>
       <c r="B33" s="10" t="str">
         <f aca="false">IF(INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A33),$L$9:$L$38,0))&lt;=0,"",INDEX($I$9:$I$38,MATCH(LARGE($L$9:$L$38,A33),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="C33" s="22" t="str">
+      <c r="C33" s="23" t="str">
         <f aca="false">IF(B33="","",INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A33),$L$9:$L$38,0)))</f>
         <v/>
       </c>
@@ -25395,40 +25529,44 @@
         <f aca="false">IF(B33="","",INDEX($K$9:$K$38,MATCH(LARGE($L$9:$L$38,A33),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="E33" s="23" t="str">
+      <c r="E33" s="24" t="str">
         <f aca="false">IF(OR(B33="",$B$6=0),"",C33/$B$6)</f>
         <v/>
       </c>
-      <c r="F33" s="23" t="str">
+      <c r="F33" s="24" t="str">
         <f aca="false">IF(OR(B33="",$B$6=0),"",SUM($C$9:C33)/$B$6)</f>
         <v/>
       </c>
-      <c r="I33" s="24" t="str">
+      <c r="I33" s="25" t="str">
         <f aca="false">IF(Setup!D29="","",IF(SUMPRODUCT(--(Setup!$D$4:D28=Setup!D29))&gt;0,"",Setup!D29))</f>
         <v/>
       </c>
-      <c r="J33" s="24" t="n">
+      <c r="J33" s="25" t="n">
         <f aca="false">IF(I33="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I33)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0),'Downtime Log'!$G$5:$G$1004))</f>
         <v>0</v>
       </c>
-      <c r="K33" s="24" t="n">
+      <c r="K33" s="25" t="n">
         <f aca="false">IF(I33="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I33)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>0</v>
       </c>
-      <c r="L33" s="24" t="n">
+      <c r="L33" s="25" t="n">
         <f aca="false">IF(I33="",-1,J33+(34-25)/1000000)</f>
         <v>-1</v>
       </c>
+      <c r="M33" s="26" t="n">
+        <f aca="false">IF(B33&lt;&gt;"",F33,M32)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="21" t="n">
+      <c r="A34" s="22" t="n">
         <v>26</v>
       </c>
       <c r="B34" s="10" t="str">
         <f aca="false">IF(INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A34),$L$9:$L$38,0))&lt;=0,"",INDEX($I$9:$I$38,MATCH(LARGE($L$9:$L$38,A34),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="C34" s="22" t="str">
+      <c r="C34" s="23" t="str">
         <f aca="false">IF(B34="","",INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A34),$L$9:$L$38,0)))</f>
         <v/>
       </c>
@@ -25436,40 +25574,44 @@
         <f aca="false">IF(B34="","",INDEX($K$9:$K$38,MATCH(LARGE($L$9:$L$38,A34),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="E34" s="23" t="str">
+      <c r="E34" s="24" t="str">
         <f aca="false">IF(OR(B34="",$B$6=0),"",C34/$B$6)</f>
         <v/>
       </c>
-      <c r="F34" s="23" t="str">
+      <c r="F34" s="24" t="str">
         <f aca="false">IF(OR(B34="",$B$6=0),"",SUM($C$9:C34)/$B$6)</f>
         <v/>
       </c>
-      <c r="I34" s="24" t="str">
+      <c r="I34" s="25" t="str">
         <f aca="false">IF(Setup!D30="","",IF(SUMPRODUCT(--(Setup!$D$4:D29=Setup!D30))&gt;0,"",Setup!D30))</f>
         <v/>
       </c>
-      <c r="J34" s="24" t="n">
+      <c r="J34" s="25" t="n">
         <f aca="false">IF(I34="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I34)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0),'Downtime Log'!$G$5:$G$1004))</f>
         <v>0</v>
       </c>
-      <c r="K34" s="24" t="n">
+      <c r="K34" s="25" t="n">
         <f aca="false">IF(I34="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I34)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>0</v>
       </c>
-      <c r="L34" s="24" t="n">
+      <c r="L34" s="25" t="n">
         <f aca="false">IF(I34="",-1,J34+(34-26)/1000000)</f>
         <v>-1</v>
       </c>
+      <c r="M34" s="26" t="n">
+        <f aca="false">IF(B34&lt;&gt;"",F34,M33)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="21" t="n">
+      <c r="A35" s="22" t="n">
         <v>27</v>
       </c>
       <c r="B35" s="10" t="str">
         <f aca="false">IF(INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A35),$L$9:$L$38,0))&lt;=0,"",INDEX($I$9:$I$38,MATCH(LARGE($L$9:$L$38,A35),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="C35" s="22" t="str">
+      <c r="C35" s="23" t="str">
         <f aca="false">IF(B35="","",INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A35),$L$9:$L$38,0)))</f>
         <v/>
       </c>
@@ -25477,40 +25619,44 @@
         <f aca="false">IF(B35="","",INDEX($K$9:$K$38,MATCH(LARGE($L$9:$L$38,A35),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="E35" s="23" t="str">
+      <c r="E35" s="24" t="str">
         <f aca="false">IF(OR(B35="",$B$6=0),"",C35/$B$6)</f>
         <v/>
       </c>
-      <c r="F35" s="23" t="str">
+      <c r="F35" s="24" t="str">
         <f aca="false">IF(OR(B35="",$B$6=0),"",SUM($C$9:C35)/$B$6)</f>
         <v/>
       </c>
-      <c r="I35" s="24" t="str">
+      <c r="I35" s="25" t="str">
         <f aca="false">IF(Setup!D31="","",IF(SUMPRODUCT(--(Setup!$D$4:D30=Setup!D31))&gt;0,"",Setup!D31))</f>
         <v/>
       </c>
-      <c r="J35" s="24" t="n">
+      <c r="J35" s="25" t="n">
         <f aca="false">IF(I35="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I35)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0),'Downtime Log'!$G$5:$G$1004))</f>
         <v>0</v>
       </c>
-      <c r="K35" s="24" t="n">
+      <c r="K35" s="25" t="n">
         <f aca="false">IF(I35="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I35)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>0</v>
       </c>
-      <c r="L35" s="24" t="n">
+      <c r="L35" s="25" t="n">
         <f aca="false">IF(I35="",-1,J35+(34-27)/1000000)</f>
         <v>-1</v>
       </c>
+      <c r="M35" s="26" t="n">
+        <f aca="false">IF(B35&lt;&gt;"",F35,M34)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="21" t="n">
+      <c r="A36" s="22" t="n">
         <v>28</v>
       </c>
       <c r="B36" s="10" t="str">
         <f aca="false">IF(INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A36),$L$9:$L$38,0))&lt;=0,"",INDEX($I$9:$I$38,MATCH(LARGE($L$9:$L$38,A36),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="C36" s="22" t="str">
+      <c r="C36" s="23" t="str">
         <f aca="false">IF(B36="","",INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A36),$L$9:$L$38,0)))</f>
         <v/>
       </c>
@@ -25518,40 +25664,44 @@
         <f aca="false">IF(B36="","",INDEX($K$9:$K$38,MATCH(LARGE($L$9:$L$38,A36),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="E36" s="23" t="str">
+      <c r="E36" s="24" t="str">
         <f aca="false">IF(OR(B36="",$B$6=0),"",C36/$B$6)</f>
         <v/>
       </c>
-      <c r="F36" s="23" t="str">
+      <c r="F36" s="24" t="str">
         <f aca="false">IF(OR(B36="",$B$6=0),"",SUM($C$9:C36)/$B$6)</f>
         <v/>
       </c>
-      <c r="I36" s="24" t="str">
+      <c r="I36" s="25" t="str">
         <f aca="false">IF(Setup!D32="","",IF(SUMPRODUCT(--(Setup!$D$4:D31=Setup!D32))&gt;0,"",Setup!D32))</f>
         <v/>
       </c>
-      <c r="J36" s="24" t="n">
+      <c r="J36" s="25" t="n">
         <f aca="false">IF(I36="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I36)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0),'Downtime Log'!$G$5:$G$1004))</f>
         <v>0</v>
       </c>
-      <c r="K36" s="24" t="n">
+      <c r="K36" s="25" t="n">
         <f aca="false">IF(I36="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I36)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>0</v>
       </c>
-      <c r="L36" s="24" t="n">
+      <c r="L36" s="25" t="n">
         <f aca="false">IF(I36="",-1,J36+(34-28)/1000000)</f>
         <v>-1</v>
       </c>
+      <c r="M36" s="26" t="n">
+        <f aca="false">IF(B36&lt;&gt;"",F36,M35)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="21" t="n">
+      <c r="A37" s="22" t="n">
         <v>29</v>
       </c>
       <c r="B37" s="10" t="str">
         <f aca="false">IF(INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A37),$L$9:$L$38,0))&lt;=0,"",INDEX($I$9:$I$38,MATCH(LARGE($L$9:$L$38,A37),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="C37" s="22" t="str">
+      <c r="C37" s="23" t="str">
         <f aca="false">IF(B37="","",INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A37),$L$9:$L$38,0)))</f>
         <v/>
       </c>
@@ -25559,40 +25709,44 @@
         <f aca="false">IF(B37="","",INDEX($K$9:$K$38,MATCH(LARGE($L$9:$L$38,A37),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="E37" s="23" t="str">
+      <c r="E37" s="24" t="str">
         <f aca="false">IF(OR(B37="",$B$6=0),"",C37/$B$6)</f>
         <v/>
       </c>
-      <c r="F37" s="23" t="str">
+      <c r="F37" s="24" t="str">
         <f aca="false">IF(OR(B37="",$B$6=0),"",SUM($C$9:C37)/$B$6)</f>
         <v/>
       </c>
-      <c r="I37" s="24" t="str">
+      <c r="I37" s="25" t="str">
         <f aca="false">IF(Setup!D33="","",IF(SUMPRODUCT(--(Setup!$D$4:D32=Setup!D33))&gt;0,"",Setup!D33))</f>
         <v/>
       </c>
-      <c r="J37" s="24" t="n">
+      <c r="J37" s="25" t="n">
         <f aca="false">IF(I37="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I37)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0),'Downtime Log'!$G$5:$G$1004))</f>
         <v>0</v>
       </c>
-      <c r="K37" s="24" t="n">
+      <c r="K37" s="25" t="n">
         <f aca="false">IF(I37="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I37)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>0</v>
       </c>
-      <c r="L37" s="24" t="n">
+      <c r="L37" s="25" t="n">
         <f aca="false">IF(I37="",-1,J37+(34-29)/1000000)</f>
         <v>-1</v>
       </c>
+      <c r="M37" s="26" t="n">
+        <f aca="false">IF(B37&lt;&gt;"",F37,M36)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="21" t="n">
+      <c r="A38" s="22" t="n">
         <v>30</v>
       </c>
       <c r="B38" s="10" t="str">
         <f aca="false">IF(INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A38),$L$9:$L$38,0))&lt;=0,"",INDEX($I$9:$I$38,MATCH(LARGE($L$9:$L$38,A38),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="C38" s="22" t="str">
+      <c r="C38" s="23" t="str">
         <f aca="false">IF(B38="","",INDEX($J$9:$J$38,MATCH(LARGE($L$9:$L$38,A38),$L$9:$L$38,0)))</f>
         <v/>
       </c>
@@ -25600,29 +25754,33 @@
         <f aca="false">IF(B38="","",INDEX($K$9:$K$38,MATCH(LARGE($L$9:$L$38,A38),$L$9:$L$38,0)))</f>
         <v/>
       </c>
-      <c r="E38" s="23" t="str">
+      <c r="E38" s="24" t="str">
         <f aca="false">IF(OR(B38="",$B$6=0),"",C38/$B$6)</f>
         <v/>
       </c>
-      <c r="F38" s="23" t="str">
+      <c r="F38" s="24" t="str">
         <f aca="false">IF(OR(B38="",$B$6=0),"",SUM($C$9:C38)/$B$6)</f>
         <v/>
       </c>
-      <c r="I38" s="24" t="str">
+      <c r="I38" s="25" t="str">
         <f aca="false">IF(Setup!D34="","",IF(SUMPRODUCT(--(Setup!$D$4:D33=Setup!D34))&gt;0,"",Setup!D34))</f>
         <v/>
       </c>
-      <c r="J38" s="24" t="n">
+      <c r="J38" s="25" t="n">
         <f aca="false">IF(I38="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I38)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0),'Downtime Log'!$G$5:$G$1004))</f>
         <v>0</v>
       </c>
-      <c r="K38" s="24" t="n">
+      <c r="K38" s="25" t="n">
         <f aca="false">IF(I38="",0,SUMPRODUCT(('Downtime Log'!$H$5:$H$1004=I38)*('Downtime Log'!$A$5:$A$1004&gt;=$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=$D$4)*((($B$5="")+('Downtime Log'!$C$5:$C$1004=$B$5))&gt;0)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>0</v>
       </c>
-      <c r="L38" s="24" t="n">
+      <c r="L38" s="25" t="n">
         <f aca="false">IF(I38="",-1,J38+(34-30)/1000000)</f>
         <v>-1</v>
+      </c>
+      <c r="M38" s="26" t="n">
+        <f aca="false">IF(B38&lt;&gt;"",F38,M37)</f>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -25690,7 +25848,7 @@
         <f aca="false">IF(Setup!A5="","",IF(SUMPRODUCT(--(Setup!$A$4:A4=Setup!A5))&gt;0,"",Setup!A5))</f>
         <v>Press 01</v>
       </c>
-      <c r="B5" s="22" t="n">
+      <c r="B5" s="23" t="n">
         <f aca="false">IF($A5="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A5)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004))</f>
         <v>105</v>
       </c>
@@ -25698,11 +25856,11 @@
         <f aca="false">IF($A5="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A5)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>3</v>
       </c>
-      <c r="D5" s="25" t="n">
+      <c r="D5" s="27" t="n">
         <f aca="false">IF(OR($A5="",N(C5)=0),"",B5/C5)</f>
         <v>35</v>
       </c>
-      <c r="E5" s="23" t="n">
+      <c r="E5" s="24" t="n">
         <f aca="false">IF(OR($A5="",$B$36=0),"",B5/$B$36)</f>
         <v>0.411764705882353</v>
       </c>
@@ -25712,7 +25870,7 @@
         <f aca="false">IF(Setup!A6="","",IF(SUMPRODUCT(--(Setup!$A$4:A5=Setup!A6))&gt;0,"",Setup!A6))</f>
         <v>CNC Lathe 02</v>
       </c>
-      <c r="B6" s="22" t="n">
+      <c r="B6" s="23" t="n">
         <f aca="false">IF($A6="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A6)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004))</f>
         <v>75</v>
       </c>
@@ -25720,11 +25878,11 @@
         <f aca="false">IF($A6="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A6)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>2</v>
       </c>
-      <c r="D6" s="25" t="n">
+      <c r="D6" s="27" t="n">
         <f aca="false">IF(OR($A6="",N(C6)=0),"",B6/C6)</f>
         <v>37.5</v>
       </c>
-      <c r="E6" s="23" t="n">
+      <c r="E6" s="24" t="n">
         <f aca="false">IF(OR($A6="",$B$36=0),"",B6/$B$36)</f>
         <v>0.294117647058824</v>
       </c>
@@ -25734,7 +25892,7 @@
         <f aca="false">IF(Setup!A7="","",IF(SUMPRODUCT(--(Setup!$A$4:A6=Setup!A7))&gt;0,"",Setup!A7))</f>
         <v>Packaging Line A</v>
       </c>
-      <c r="B7" s="22" t="n">
+      <c r="B7" s="23" t="n">
         <f aca="false">IF($A7="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A7)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004))</f>
         <v>75</v>
       </c>
@@ -25742,11 +25900,11 @@
         <f aca="false">IF($A7="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A7)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v>2</v>
       </c>
-      <c r="D7" s="25" t="n">
+      <c r="D7" s="27" t="n">
         <f aca="false">IF(OR($A7="",N(C7)=0),"",B7/C7)</f>
         <v>37.5</v>
       </c>
-      <c r="E7" s="23" t="n">
+      <c r="E7" s="24" t="n">
         <f aca="false">IF(OR($A7="",$B$36=0),"",B7/$B$36)</f>
         <v>0.294117647058824</v>
       </c>
@@ -25756,7 +25914,7 @@
         <f aca="false">IF(Setup!A8="","",IF(SUMPRODUCT(--(Setup!$A$4:A7=Setup!A8))&gt;0,"",Setup!A8))</f>
         <v/>
       </c>
-      <c r="B8" s="22" t="str">
+      <c r="B8" s="23" t="str">
         <f aca="false">IF($A8="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A8)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004))</f>
         <v/>
       </c>
@@ -25764,11 +25922,11 @@
         <f aca="false">IF($A8="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A8)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v/>
       </c>
-      <c r="D8" s="25" t="str">
+      <c r="D8" s="27" t="str">
         <f aca="false">IF(OR($A8="",N(C8)=0),"",B8/C8)</f>
         <v/>
       </c>
-      <c r="E8" s="23" t="str">
+      <c r="E8" s="24" t="str">
         <f aca="false">IF(OR($A8="",$B$36=0),"",B8/$B$36)</f>
         <v/>
       </c>
@@ -25778,7 +25936,7 @@
         <f aca="false">IF(Setup!A9="","",IF(SUMPRODUCT(--(Setup!$A$4:A8=Setup!A9))&gt;0,"",Setup!A9))</f>
         <v/>
       </c>
-      <c r="B9" s="22" t="str">
+      <c r="B9" s="23" t="str">
         <f aca="false">IF($A9="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A9)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004))</f>
         <v/>
       </c>
@@ -25786,11 +25944,11 @@
         <f aca="false">IF($A9="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A9)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v/>
       </c>
-      <c r="D9" s="25" t="str">
+      <c r="D9" s="27" t="str">
         <f aca="false">IF(OR($A9="",N(C9)=0),"",B9/C9)</f>
         <v/>
       </c>
-      <c r="E9" s="23" t="str">
+      <c r="E9" s="24" t="str">
         <f aca="false">IF(OR($A9="",$B$36=0),"",B9/$B$36)</f>
         <v/>
       </c>
@@ -25800,7 +25958,7 @@
         <f aca="false">IF(Setup!A10="","",IF(SUMPRODUCT(--(Setup!$A$4:A9=Setup!A10))&gt;0,"",Setup!A10))</f>
         <v/>
       </c>
-      <c r="B10" s="22" t="str">
+      <c r="B10" s="23" t="str">
         <f aca="false">IF($A10="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A10)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004))</f>
         <v/>
       </c>
@@ -25808,11 +25966,11 @@
         <f aca="false">IF($A10="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A10)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v/>
       </c>
-      <c r="D10" s="25" t="str">
+      <c r="D10" s="27" t="str">
         <f aca="false">IF(OR($A10="",N(C10)=0),"",B10/C10)</f>
         <v/>
       </c>
-      <c r="E10" s="23" t="str">
+      <c r="E10" s="24" t="str">
         <f aca="false">IF(OR($A10="",$B$36=0),"",B10/$B$36)</f>
         <v/>
       </c>
@@ -25822,7 +25980,7 @@
         <f aca="false">IF(Setup!A11="","",IF(SUMPRODUCT(--(Setup!$A$4:A10=Setup!A11))&gt;0,"",Setup!A11))</f>
         <v/>
       </c>
-      <c r="B11" s="22" t="str">
+      <c r="B11" s="23" t="str">
         <f aca="false">IF($A11="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A11)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004))</f>
         <v/>
       </c>
@@ -25830,11 +25988,11 @@
         <f aca="false">IF($A11="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A11)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v/>
       </c>
-      <c r="D11" s="25" t="str">
+      <c r="D11" s="27" t="str">
         <f aca="false">IF(OR($A11="",N(C11)=0),"",B11/C11)</f>
         <v/>
       </c>
-      <c r="E11" s="23" t="str">
+      <c r="E11" s="24" t="str">
         <f aca="false">IF(OR($A11="",$B$36=0),"",B11/$B$36)</f>
         <v/>
       </c>
@@ -25844,7 +26002,7 @@
         <f aca="false">IF(Setup!A12="","",IF(SUMPRODUCT(--(Setup!$A$4:A11=Setup!A12))&gt;0,"",Setup!A12))</f>
         <v/>
       </c>
-      <c r="B12" s="22" t="str">
+      <c r="B12" s="23" t="str">
         <f aca="false">IF($A12="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A12)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004))</f>
         <v/>
       </c>
@@ -25852,11 +26010,11 @@
         <f aca="false">IF($A12="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A12)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v/>
       </c>
-      <c r="D12" s="25" t="str">
+      <c r="D12" s="27" t="str">
         <f aca="false">IF(OR($A12="",N(C12)=0),"",B12/C12)</f>
         <v/>
       </c>
-      <c r="E12" s="23" t="str">
+      <c r="E12" s="24" t="str">
         <f aca="false">IF(OR($A12="",$B$36=0),"",B12/$B$36)</f>
         <v/>
       </c>
@@ -25866,7 +26024,7 @@
         <f aca="false">IF(Setup!A13="","",IF(SUMPRODUCT(--(Setup!$A$4:A12=Setup!A13))&gt;0,"",Setup!A13))</f>
         <v/>
       </c>
-      <c r="B13" s="22" t="str">
+      <c r="B13" s="23" t="str">
         <f aca="false">IF($A13="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A13)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004))</f>
         <v/>
       </c>
@@ -25874,11 +26032,11 @@
         <f aca="false">IF($A13="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A13)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v/>
       </c>
-      <c r="D13" s="25" t="str">
+      <c r="D13" s="27" t="str">
         <f aca="false">IF(OR($A13="",N(C13)=0),"",B13/C13)</f>
         <v/>
       </c>
-      <c r="E13" s="23" t="str">
+      <c r="E13" s="24" t="str">
         <f aca="false">IF(OR($A13="",$B$36=0),"",B13/$B$36)</f>
         <v/>
       </c>
@@ -25888,7 +26046,7 @@
         <f aca="false">IF(Setup!A14="","",IF(SUMPRODUCT(--(Setup!$A$4:A13=Setup!A14))&gt;0,"",Setup!A14))</f>
         <v/>
       </c>
-      <c r="B14" s="22" t="str">
+      <c r="B14" s="23" t="str">
         <f aca="false">IF($A14="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A14)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004))</f>
         <v/>
       </c>
@@ -25896,11 +26054,11 @@
         <f aca="false">IF($A14="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A14)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v/>
       </c>
-      <c r="D14" s="25" t="str">
+      <c r="D14" s="27" t="str">
         <f aca="false">IF(OR($A14="",N(C14)=0),"",B14/C14)</f>
         <v/>
       </c>
-      <c r="E14" s="23" t="str">
+      <c r="E14" s="24" t="str">
         <f aca="false">IF(OR($A14="",$B$36=0),"",B14/$B$36)</f>
         <v/>
       </c>
@@ -25910,7 +26068,7 @@
         <f aca="false">IF(Setup!A15="","",IF(SUMPRODUCT(--(Setup!$A$4:A14=Setup!A15))&gt;0,"",Setup!A15))</f>
         <v/>
       </c>
-      <c r="B15" s="22" t="str">
+      <c r="B15" s="23" t="str">
         <f aca="false">IF($A15="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A15)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004))</f>
         <v/>
       </c>
@@ -25918,11 +26076,11 @@
         <f aca="false">IF($A15="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A15)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v/>
       </c>
-      <c r="D15" s="25" t="str">
+      <c r="D15" s="27" t="str">
         <f aca="false">IF(OR($A15="",N(C15)=0),"",B15/C15)</f>
         <v/>
       </c>
-      <c r="E15" s="23" t="str">
+      <c r="E15" s="24" t="str">
         <f aca="false">IF(OR($A15="",$B$36=0),"",B15/$B$36)</f>
         <v/>
       </c>
@@ -25932,7 +26090,7 @@
         <f aca="false">IF(Setup!A16="","",IF(SUMPRODUCT(--(Setup!$A$4:A15=Setup!A16))&gt;0,"",Setup!A16))</f>
         <v/>
       </c>
-      <c r="B16" s="22" t="str">
+      <c r="B16" s="23" t="str">
         <f aca="false">IF($A16="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A16)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004))</f>
         <v/>
       </c>
@@ -25940,11 +26098,11 @@
         <f aca="false">IF($A16="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A16)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v/>
       </c>
-      <c r="D16" s="25" t="str">
+      <c r="D16" s="27" t="str">
         <f aca="false">IF(OR($A16="",N(C16)=0),"",B16/C16)</f>
         <v/>
       </c>
-      <c r="E16" s="23" t="str">
+      <c r="E16" s="24" t="str">
         <f aca="false">IF(OR($A16="",$B$36=0),"",B16/$B$36)</f>
         <v/>
       </c>
@@ -25954,7 +26112,7 @@
         <f aca="false">IF(Setup!A17="","",IF(SUMPRODUCT(--(Setup!$A$4:A16=Setup!A17))&gt;0,"",Setup!A17))</f>
         <v/>
       </c>
-      <c r="B17" s="22" t="str">
+      <c r="B17" s="23" t="str">
         <f aca="false">IF($A17="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A17)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004))</f>
         <v/>
       </c>
@@ -25962,11 +26120,11 @@
         <f aca="false">IF($A17="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A17)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v/>
       </c>
-      <c r="D17" s="25" t="str">
+      <c r="D17" s="27" t="str">
         <f aca="false">IF(OR($A17="",N(C17)=0),"",B17/C17)</f>
         <v/>
       </c>
-      <c r="E17" s="23" t="str">
+      <c r="E17" s="24" t="str">
         <f aca="false">IF(OR($A17="",$B$36=0),"",B17/$B$36)</f>
         <v/>
       </c>
@@ -25976,7 +26134,7 @@
         <f aca="false">IF(Setup!A18="","",IF(SUMPRODUCT(--(Setup!$A$4:A17=Setup!A18))&gt;0,"",Setup!A18))</f>
         <v/>
       </c>
-      <c r="B18" s="22" t="str">
+      <c r="B18" s="23" t="str">
         <f aca="false">IF($A18="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A18)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004))</f>
         <v/>
       </c>
@@ -25984,11 +26142,11 @@
         <f aca="false">IF($A18="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A18)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v/>
       </c>
-      <c r="D18" s="25" t="str">
+      <c r="D18" s="27" t="str">
         <f aca="false">IF(OR($A18="",N(C18)=0),"",B18/C18)</f>
         <v/>
       </c>
-      <c r="E18" s="23" t="str">
+      <c r="E18" s="24" t="str">
         <f aca="false">IF(OR($A18="",$B$36=0),"",B18/$B$36)</f>
         <v/>
       </c>
@@ -25998,7 +26156,7 @@
         <f aca="false">IF(Setup!A19="","",IF(SUMPRODUCT(--(Setup!$A$4:A18=Setup!A19))&gt;0,"",Setup!A19))</f>
         <v/>
       </c>
-      <c r="B19" s="22" t="str">
+      <c r="B19" s="23" t="str">
         <f aca="false">IF($A19="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A19)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004))</f>
         <v/>
       </c>
@@ -26006,11 +26164,11 @@
         <f aca="false">IF($A19="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A19)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v/>
       </c>
-      <c r="D19" s="25" t="str">
+      <c r="D19" s="27" t="str">
         <f aca="false">IF(OR($A19="",N(C19)=0),"",B19/C19)</f>
         <v/>
       </c>
-      <c r="E19" s="23" t="str">
+      <c r="E19" s="24" t="str">
         <f aca="false">IF(OR($A19="",$B$36=0),"",B19/$B$36)</f>
         <v/>
       </c>
@@ -26020,7 +26178,7 @@
         <f aca="false">IF(Setup!A20="","",IF(SUMPRODUCT(--(Setup!$A$4:A19=Setup!A20))&gt;0,"",Setup!A20))</f>
         <v/>
       </c>
-      <c r="B20" s="22" t="str">
+      <c r="B20" s="23" t="str">
         <f aca="false">IF($A20="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A20)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004))</f>
         <v/>
       </c>
@@ -26028,11 +26186,11 @@
         <f aca="false">IF($A20="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A20)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v/>
       </c>
-      <c r="D20" s="25" t="str">
+      <c r="D20" s="27" t="str">
         <f aca="false">IF(OR($A20="",N(C20)=0),"",B20/C20)</f>
         <v/>
       </c>
-      <c r="E20" s="23" t="str">
+      <c r="E20" s="24" t="str">
         <f aca="false">IF(OR($A20="",$B$36=0),"",B20/$B$36)</f>
         <v/>
       </c>
@@ -26042,7 +26200,7 @@
         <f aca="false">IF(Setup!A21="","",IF(SUMPRODUCT(--(Setup!$A$4:A20=Setup!A21))&gt;0,"",Setup!A21))</f>
         <v/>
       </c>
-      <c r="B21" s="22" t="str">
+      <c r="B21" s="23" t="str">
         <f aca="false">IF($A21="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A21)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004))</f>
         <v/>
       </c>
@@ -26050,11 +26208,11 @@
         <f aca="false">IF($A21="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A21)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v/>
       </c>
-      <c r="D21" s="25" t="str">
+      <c r="D21" s="27" t="str">
         <f aca="false">IF(OR($A21="",N(C21)=0),"",B21/C21)</f>
         <v/>
       </c>
-      <c r="E21" s="23" t="str">
+      <c r="E21" s="24" t="str">
         <f aca="false">IF(OR($A21="",$B$36=0),"",B21/$B$36)</f>
         <v/>
       </c>
@@ -26064,7 +26222,7 @@
         <f aca="false">IF(Setup!A22="","",IF(SUMPRODUCT(--(Setup!$A$4:A21=Setup!A22))&gt;0,"",Setup!A22))</f>
         <v/>
       </c>
-      <c r="B22" s="22" t="str">
+      <c r="B22" s="23" t="str">
         <f aca="false">IF($A22="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A22)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004))</f>
         <v/>
       </c>
@@ -26072,11 +26230,11 @@
         <f aca="false">IF($A22="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A22)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v/>
       </c>
-      <c r="D22" s="25" t="str">
+      <c r="D22" s="27" t="str">
         <f aca="false">IF(OR($A22="",N(C22)=0),"",B22/C22)</f>
         <v/>
       </c>
-      <c r="E22" s="23" t="str">
+      <c r="E22" s="24" t="str">
         <f aca="false">IF(OR($A22="",$B$36=0),"",B22/$B$36)</f>
         <v/>
       </c>
@@ -26086,7 +26244,7 @@
         <f aca="false">IF(Setup!A23="","",IF(SUMPRODUCT(--(Setup!$A$4:A22=Setup!A23))&gt;0,"",Setup!A23))</f>
         <v/>
       </c>
-      <c r="B23" s="22" t="str">
+      <c r="B23" s="23" t="str">
         <f aca="false">IF($A23="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A23)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004))</f>
         <v/>
       </c>
@@ -26094,11 +26252,11 @@
         <f aca="false">IF($A23="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A23)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v/>
       </c>
-      <c r="D23" s="25" t="str">
+      <c r="D23" s="27" t="str">
         <f aca="false">IF(OR($A23="",N(C23)=0),"",B23/C23)</f>
         <v/>
       </c>
-      <c r="E23" s="23" t="str">
+      <c r="E23" s="24" t="str">
         <f aca="false">IF(OR($A23="",$B$36=0),"",B23/$B$36)</f>
         <v/>
       </c>
@@ -26108,7 +26266,7 @@
         <f aca="false">IF(Setup!A24="","",IF(SUMPRODUCT(--(Setup!$A$4:A23=Setup!A24))&gt;0,"",Setup!A24))</f>
         <v/>
       </c>
-      <c r="B24" s="22" t="str">
+      <c r="B24" s="23" t="str">
         <f aca="false">IF($A24="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A24)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004))</f>
         <v/>
       </c>
@@ -26116,11 +26274,11 @@
         <f aca="false">IF($A24="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A24)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v/>
       </c>
-      <c r="D24" s="25" t="str">
+      <c r="D24" s="27" t="str">
         <f aca="false">IF(OR($A24="",N(C24)=0),"",B24/C24)</f>
         <v/>
       </c>
-      <c r="E24" s="23" t="str">
+      <c r="E24" s="24" t="str">
         <f aca="false">IF(OR($A24="",$B$36=0),"",B24/$B$36)</f>
         <v/>
       </c>
@@ -26130,7 +26288,7 @@
         <f aca="false">IF(Setup!A25="","",IF(SUMPRODUCT(--(Setup!$A$4:A24=Setup!A25))&gt;0,"",Setup!A25))</f>
         <v/>
       </c>
-      <c r="B25" s="22" t="str">
+      <c r="B25" s="23" t="str">
         <f aca="false">IF($A25="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A25)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004))</f>
         <v/>
       </c>
@@ -26138,11 +26296,11 @@
         <f aca="false">IF($A25="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A25)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v/>
       </c>
-      <c r="D25" s="25" t="str">
+      <c r="D25" s="27" t="str">
         <f aca="false">IF(OR($A25="",N(C25)=0),"",B25/C25)</f>
         <v/>
       </c>
-      <c r="E25" s="23" t="str">
+      <c r="E25" s="24" t="str">
         <f aca="false">IF(OR($A25="",$B$36=0),"",B25/$B$36)</f>
         <v/>
       </c>
@@ -26152,7 +26310,7 @@
         <f aca="false">IF(Setup!A26="","",IF(SUMPRODUCT(--(Setup!$A$4:A25=Setup!A26))&gt;0,"",Setup!A26))</f>
         <v/>
       </c>
-      <c r="B26" s="22" t="str">
+      <c r="B26" s="23" t="str">
         <f aca="false">IF($A26="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A26)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004))</f>
         <v/>
       </c>
@@ -26160,11 +26318,11 @@
         <f aca="false">IF($A26="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A26)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v/>
       </c>
-      <c r="D26" s="25" t="str">
+      <c r="D26" s="27" t="str">
         <f aca="false">IF(OR($A26="",N(C26)=0),"",B26/C26)</f>
         <v/>
       </c>
-      <c r="E26" s="23" t="str">
+      <c r="E26" s="24" t="str">
         <f aca="false">IF(OR($A26="",$B$36=0),"",B26/$B$36)</f>
         <v/>
       </c>
@@ -26174,7 +26332,7 @@
         <f aca="false">IF(Setup!A27="","",IF(SUMPRODUCT(--(Setup!$A$4:A26=Setup!A27))&gt;0,"",Setup!A27))</f>
         <v/>
       </c>
-      <c r="B27" s="22" t="str">
+      <c r="B27" s="23" t="str">
         <f aca="false">IF($A27="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A27)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004))</f>
         <v/>
       </c>
@@ -26182,11 +26340,11 @@
         <f aca="false">IF($A27="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A27)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v/>
       </c>
-      <c r="D27" s="25" t="str">
+      <c r="D27" s="27" t="str">
         <f aca="false">IF(OR($A27="",N(C27)=0),"",B27/C27)</f>
         <v/>
       </c>
-      <c r="E27" s="23" t="str">
+      <c r="E27" s="24" t="str">
         <f aca="false">IF(OR($A27="",$B$36=0),"",B27/$B$36)</f>
         <v/>
       </c>
@@ -26196,7 +26354,7 @@
         <f aca="false">IF(Setup!A28="","",IF(SUMPRODUCT(--(Setup!$A$4:A27=Setup!A28))&gt;0,"",Setup!A28))</f>
         <v/>
       </c>
-      <c r="B28" s="22" t="str">
+      <c r="B28" s="23" t="str">
         <f aca="false">IF($A28="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A28)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004))</f>
         <v/>
       </c>
@@ -26204,11 +26362,11 @@
         <f aca="false">IF($A28="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A28)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v/>
       </c>
-      <c r="D28" s="25" t="str">
+      <c r="D28" s="27" t="str">
         <f aca="false">IF(OR($A28="",N(C28)=0),"",B28/C28)</f>
         <v/>
       </c>
-      <c r="E28" s="23" t="str">
+      <c r="E28" s="24" t="str">
         <f aca="false">IF(OR($A28="",$B$36=0),"",B28/$B$36)</f>
         <v/>
       </c>
@@ -26218,7 +26376,7 @@
         <f aca="false">IF(Setup!A29="","",IF(SUMPRODUCT(--(Setup!$A$4:A28=Setup!A29))&gt;0,"",Setup!A29))</f>
         <v/>
       </c>
-      <c r="B29" s="22" t="str">
+      <c r="B29" s="23" t="str">
         <f aca="false">IF($A29="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A29)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004))</f>
         <v/>
       </c>
@@ -26226,11 +26384,11 @@
         <f aca="false">IF($A29="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A29)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v/>
       </c>
-      <c r="D29" s="25" t="str">
+      <c r="D29" s="27" t="str">
         <f aca="false">IF(OR($A29="",N(C29)=0),"",B29/C29)</f>
         <v/>
       </c>
-      <c r="E29" s="23" t="str">
+      <c r="E29" s="24" t="str">
         <f aca="false">IF(OR($A29="",$B$36=0),"",B29/$B$36)</f>
         <v/>
       </c>
@@ -26240,7 +26398,7 @@
         <f aca="false">IF(Setup!A30="","",IF(SUMPRODUCT(--(Setup!$A$4:A29=Setup!A30))&gt;0,"",Setup!A30))</f>
         <v/>
       </c>
-      <c r="B30" s="22" t="str">
+      <c r="B30" s="23" t="str">
         <f aca="false">IF($A30="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A30)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004))</f>
         <v/>
       </c>
@@ -26248,11 +26406,11 @@
         <f aca="false">IF($A30="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A30)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v/>
       </c>
-      <c r="D30" s="25" t="str">
+      <c r="D30" s="27" t="str">
         <f aca="false">IF(OR($A30="",N(C30)=0),"",B30/C30)</f>
         <v/>
       </c>
-      <c r="E30" s="23" t="str">
+      <c r="E30" s="24" t="str">
         <f aca="false">IF(OR($A30="",$B$36=0),"",B30/$B$36)</f>
         <v/>
       </c>
@@ -26262,7 +26420,7 @@
         <f aca="false">IF(Setup!A31="","",IF(SUMPRODUCT(--(Setup!$A$4:A30=Setup!A31))&gt;0,"",Setup!A31))</f>
         <v/>
       </c>
-      <c r="B31" s="22" t="str">
+      <c r="B31" s="23" t="str">
         <f aca="false">IF($A31="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A31)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004))</f>
         <v/>
       </c>
@@ -26270,11 +26428,11 @@
         <f aca="false">IF($A31="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A31)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v/>
       </c>
-      <c r="D31" s="25" t="str">
+      <c r="D31" s="27" t="str">
         <f aca="false">IF(OR($A31="",N(C31)=0),"",B31/C31)</f>
         <v/>
       </c>
-      <c r="E31" s="23" t="str">
+      <c r="E31" s="24" t="str">
         <f aca="false">IF(OR($A31="",$B$36=0),"",B31/$B$36)</f>
         <v/>
       </c>
@@ -26284,7 +26442,7 @@
         <f aca="false">IF(Setup!A32="","",IF(SUMPRODUCT(--(Setup!$A$4:A31=Setup!A32))&gt;0,"",Setup!A32))</f>
         <v/>
       </c>
-      <c r="B32" s="22" t="str">
+      <c r="B32" s="23" t="str">
         <f aca="false">IF($A32="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A32)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004))</f>
         <v/>
       </c>
@@ -26292,11 +26450,11 @@
         <f aca="false">IF($A32="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A32)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v/>
       </c>
-      <c r="D32" s="25" t="str">
+      <c r="D32" s="27" t="str">
         <f aca="false">IF(OR($A32="",N(C32)=0),"",B32/C32)</f>
         <v/>
       </c>
-      <c r="E32" s="23" t="str">
+      <c r="E32" s="24" t="str">
         <f aca="false">IF(OR($A32="",$B$36=0),"",B32/$B$36)</f>
         <v/>
       </c>
@@ -26306,7 +26464,7 @@
         <f aca="false">IF(Setup!A33="","",IF(SUMPRODUCT(--(Setup!$A$4:A32=Setup!A33))&gt;0,"",Setup!A33))</f>
         <v/>
       </c>
-      <c r="B33" s="22" t="str">
+      <c r="B33" s="23" t="str">
         <f aca="false">IF($A33="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A33)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004))</f>
         <v/>
       </c>
@@ -26314,11 +26472,11 @@
         <f aca="false">IF($A33="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A33)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v/>
       </c>
-      <c r="D33" s="25" t="str">
+      <c r="D33" s="27" t="str">
         <f aca="false">IF(OR($A33="",N(C33)=0),"",B33/C33)</f>
         <v/>
       </c>
-      <c r="E33" s="23" t="str">
+      <c r="E33" s="24" t="str">
         <f aca="false">IF(OR($A33="",$B$36=0),"",B33/$B$36)</f>
         <v/>
       </c>
@@ -26328,7 +26486,7 @@
         <f aca="false">IF(Setup!A34="","",IF(SUMPRODUCT(--(Setup!$A$4:A33=Setup!A34))&gt;0,"",Setup!A34))</f>
         <v/>
       </c>
-      <c r="B34" s="22" t="str">
+      <c r="B34" s="23" t="str">
         <f aca="false">IF($A34="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A34)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004))</f>
         <v/>
       </c>
@@ -26336,11 +26494,11 @@
         <f aca="false">IF($A34="","",SUMPRODUCT(('Downtime Log'!$C$5:$C$1004=$A34)*('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0)))</f>
         <v/>
       </c>
-      <c r="D34" s="25" t="str">
+      <c r="D34" s="27" t="str">
         <f aca="false">IF(OR($A34="",N(C34)=0),"",B34/C34)</f>
         <v/>
       </c>
-      <c r="E34" s="23" t="str">
+      <c r="E34" s="24" t="str">
         <f aca="false">IF(OR($A34="",$B$36=0),"",B34/$B$36)</f>
         <v/>
       </c>
@@ -26349,7 +26507,7 @@
       <c r="A35" s="10" t="s">
         <v>84</v>
       </c>
-      <c r="B35" s="22" t="n">
+      <c r="B35" s="23" t="n">
         <f aca="false">B36-SUM(B5:B34)</f>
         <v>0</v>
       </c>
@@ -26357,32 +26515,32 @@
         <f aca="false">SUMPRODUCT(('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0))-SUM(C5:C34)</f>
         <v>0</v>
       </c>
-      <c r="D35" s="25" t="str">
+      <c r="D35" s="27" t="str">
         <f aca="false">IF(OR($A35="",N(C35)=0),"",B35/C35)</f>
         <v/>
       </c>
-      <c r="E35" s="23" t="n">
+      <c r="E35" s="24" t="n">
         <f aca="false">IF(OR($A35="",$B$36=0),"",B35/$B$36)</f>
         <v>0</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="26" t="s">
+      <c r="A36" s="28" t="s">
         <v>85</v>
       </c>
-      <c r="B36" s="27" t="n">
+      <c r="B36" s="29" t="n">
         <f aca="false">SUMPRODUCT(('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4),'Downtime Log'!$G$5:$G$1004)</f>
         <v>255</v>
       </c>
-      <c r="C36" s="28" t="n">
+      <c r="C36" s="30" t="n">
         <f aca="false">SUMPRODUCT(('Downtime Log'!$A$5:$A$1004&gt;=Pareto!$D$3)*('Downtime Log'!$A$5:$A$1004&lt;=Pareto!$D$4)*ISNUMBER('Downtime Log'!$G$5:$G$1004)*('Downtime Log'!$G$5:$G$1004&gt;0))</f>
         <v>7</v>
       </c>
-      <c r="D36" s="29" t="n">
+      <c r="D36" s="31" t="n">
         <f aca="false">IF(OR($A36="",N(C36)=0),"",B36/C36)</f>
         <v>36.4285714285714</v>
       </c>
-      <c r="E36" s="30" t="n">
+      <c r="E36" s="32" t="n">
         <f aca="false">IF(OR($A36="",$B$36=0),"",B36/$B$36)</f>
         <v>1</v>
       </c>

</xml_diff>